<commit_message>
feat: multi-client testing, retry mechanism, headless mode, debug logging, remove ExcelLogger dependency
</commit_message>
<xml_diff>
--- a/src/main/resources/testdata.xlsx
+++ b/src/main/resources/testdata.xlsx
@@ -9,17 +9,18 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7500"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7500" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="TestData" sheetId="1" r:id="rId1"/>
+    <sheet name="Clients" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="60">
   <si>
     <t>Key</t>
   </si>
@@ -54,103 +55,151 @@
     <t>product.horizon</t>
   </si>
   <si>
+    <t>product.current.value</t>
+  </si>
+  <si>
+    <t>₹ 0</t>
+  </si>
+  <si>
+    <t>product.inception.date</t>
+  </si>
+  <si>
+    <t>product.benchmark</t>
+  </si>
+  <si>
+    <t>product.methodology</t>
+  </si>
+  <si>
+    <t>Fundamental</t>
+  </si>
+  <si>
+    <t>product.no.of.stocks</t>
+  </si>
+  <si>
+    <t>15-20</t>
+  </si>
+  <si>
+    <t>activation.model.description</t>
+  </si>
+  <si>
+    <t>A concentrated portfolio that blends tactical bets with long term winners.</t>
+  </si>
+  <si>
+    <t>activation.model.brokerage.standard</t>
+  </si>
+  <si>
+    <t>Standard Brokerage 1 %</t>
+  </si>
+  <si>
+    <t>activation.model.next.cta.text</t>
+  </si>
+  <si>
+    <t>Next</t>
+  </si>
+  <si>
+    <t>subscription.amount.expected</t>
+  </si>
+  <si>
+    <t>₹0</t>
+  </si>
+  <si>
+    <t>gst.amount.expected</t>
+  </si>
+  <si>
+    <t>required.margin.expected</t>
+  </si>
+  <si>
+    <t>available.amount.expected</t>
+  </si>
+  <si>
+    <t>₹5,00,00,000</t>
+  </si>
+  <si>
+    <t>invalid.amount.not.multiple</t>
+  </si>
+  <si>
+    <t>500</t>
+  </si>
+  <si>
+    <t>invalid.amount.zero</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>error.not.multiple</t>
+  </si>
+  <si>
+    <t>Investment amount should be in multiple of 1,000</t>
+  </si>
+  <si>
+    <t>error.min.amount</t>
+  </si>
+  <si>
+    <t>Please enter minimum investment amount ₹ 1,00,000</t>
+  </si>
+  <si>
+    <t>Nifty 200</t>
+  </si>
+  <si>
+    <t>app.page.title</t>
+  </si>
+  <si>
+    <t>Motilal Oswal IMP</t>
+  </si>
+  <si>
+    <t>01 Feb 21</t>
+  </si>
+  <si>
     <t>3-5 Years</t>
   </si>
   <si>
-    <t>product.current.value</t>
-  </si>
-  <si>
-    <t>₹ 0</t>
-  </si>
-  <si>
-    <t>product.inception.date</t>
-  </si>
-  <si>
-    <t>product.benchmark</t>
-  </si>
-  <si>
-    <t>product.methodology</t>
-  </si>
-  <si>
-    <t>Fundamental</t>
-  </si>
-  <si>
-    <t>product.no.of.stocks</t>
-  </si>
-  <si>
-    <t>15-20</t>
-  </si>
-  <si>
-    <t>activation.model.description</t>
-  </si>
-  <si>
-    <t>A concentrated portfolio that blends tactical bets with long term winners.</t>
-  </si>
-  <si>
-    <t>activation.model.brokerage.standard</t>
-  </si>
-  <si>
-    <t>Standard Brokerage 1 %</t>
-  </si>
-  <si>
-    <t>activation.model.next.cta.text</t>
-  </si>
-  <si>
-    <t>Next</t>
-  </si>
-  <si>
-    <t>subscription.amount.expected</t>
-  </si>
-  <si>
-    <t>₹0</t>
-  </si>
-  <si>
-    <t>gst.amount.expected</t>
-  </si>
-  <si>
-    <t>required.margin.expected</t>
-  </si>
-  <si>
-    <t>available.amount.expected</t>
-  </si>
-  <si>
-    <t>₹5,00,00,000</t>
-  </si>
-  <si>
-    <t>invalid.amount.not.multiple</t>
-  </si>
-  <si>
-    <t>500</t>
-  </si>
-  <si>
-    <t>invalid.amount.zero</t>
-  </si>
-  <si>
-    <t>0</t>
-  </si>
-  <si>
-    <t>error.not.multiple</t>
-  </si>
-  <si>
-    <t>Investment amount should be in multiple of 1,000</t>
-  </si>
-  <si>
-    <t>error.min.amount</t>
-  </si>
-  <si>
-    <t>Please enter minimum investment amount ₹ 1,00,000</t>
-  </si>
-  <si>
-    <t>Nifty 200</t>
-  </si>
-  <si>
-    <t>app.page.title</t>
-  </si>
-  <si>
-    <t>Motilal Oswal IMP</t>
-  </si>
-  <si>
-    <t>01 Feb 21</t>
+    <t>AdvisorId</t>
+  </si>
+  <si>
+    <t>AdvisorPassword</t>
+  </si>
+  <si>
+    <t>ClientCode</t>
+  </si>
+  <si>
+    <t>ProductCode</t>
+  </si>
+  <si>
+    <t>ProductName</t>
+  </si>
+  <si>
+    <t>ProductTab</t>
+  </si>
+  <si>
+    <t>MinInvestment</t>
+  </si>
+  <si>
+    <t>Multiplier</t>
+  </si>
+  <si>
+    <t>IAP@123</t>
+  </si>
+  <si>
+    <t>New Launches</t>
+  </si>
+  <si>
+    <t>ME</t>
+  </si>
+  <si>
+    <t>MO Signature Model Portfolio</t>
+  </si>
+  <si>
+    <t>Cbos@123</t>
+  </si>
+  <si>
+    <t>RFI2550</t>
+  </si>
+  <si>
+    <t>REX1324</t>
+  </si>
+  <si>
+    <t>₹2,50,000</t>
   </si>
 </sst>
 </file>
@@ -498,10 +547,10 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>41</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="60" x14ac:dyDescent="0.25">
@@ -541,139 +590,238 @@
         <v>10</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>11</v>
+        <v>43</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>12</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>16</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12" s="1" t="s">
         <v>18</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B13" s="1" t="s">
         <v>20</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B14" s="1" t="s">
         <v>22</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B15" s="1" t="s">
         <v>24</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>26</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B19" s="1" t="s">
         <v>30</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B20" s="1" t="s">
         <v>32</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B21" s="1" t="s">
         <v>34</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B22" s="1" t="s">
         <v>36</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B23" s="1" t="s">
         <v>38</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>39</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="28" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F1" t="s">
+        <v>49</v>
+      </c>
+      <c r="G1" t="s">
+        <v>50</v>
+      </c>
+      <c r="H1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>28135</v>
+      </c>
+      <c r="B2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C2" t="s">
+        <v>57</v>
+      </c>
+      <c r="D2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F2" t="s">
+        <v>53</v>
+      </c>
+      <c r="G2" t="s">
+        <v>9</v>
+      </c>
+      <c r="H2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>40445</v>
+      </c>
+      <c r="B3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C3" t="s">
+        <v>58</v>
+      </c>
+      <c r="D3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E3" t="s">
+        <v>55</v>
+      </c>
+      <c r="F3" t="s">
+        <v>53</v>
+      </c>
+      <c r="G3" t="s">
+        <v>59</v>
+      </c>
+      <c r="H3">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
chore: update config, testdata, investment page, learning roadmap docs
</commit_message>
<xml_diff>
--- a/src/main/resources/testdata.xlsx
+++ b/src/main/resources/testdata.xlsx
@@ -3,24 +3,21 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="164011"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tejaspatil\eclipse-workspace1\selenium-framework\src\main\resources\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7500" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="17670" windowHeight="5400" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="TestData" sheetId="1" r:id="rId1"/>
     <sheet name="Clients" sheetId="2" r:id="rId2"/>
+    <sheet name="BulkClients" r:id="rId7" sheetId="3"/>
   </sheets>
   <calcPr calcId="0"/>
+  <oleSize ref="A1:Q16"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11431" uniqueCount="539">
   <si>
     <t>Key</t>
   </si>
@@ -200,13 +197,1451 @@
   </si>
   <si>
     <t>₹2,50,000</t>
+  </si>
+  <si>
+    <t>DOB</t>
+  </si>
+  <si>
+    <t>FormattedDOB</t>
+  </si>
+  <si>
+    <t>ClientType</t>
+  </si>
+  <si>
+    <t>POAStatus</t>
+  </si>
+  <si>
+    <t>IND</t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>AIM1830</t>
+  </si>
+  <si>
+    <t>1992-01-04</t>
+  </si>
+  <si>
+    <t>04/01/1992</t>
+  </si>
+  <si>
+    <t>AJIN1221</t>
+  </si>
+  <si>
+    <t>1990-12-03</t>
+  </si>
+  <si>
+    <t>03/12/1990</t>
+  </si>
+  <si>
+    <t>Akcb1448</t>
+  </si>
+  <si>
+    <t>1993-12-30</t>
+  </si>
+  <si>
+    <t>30/12/1993</t>
+  </si>
+  <si>
+    <t>AKGA1203</t>
+  </si>
+  <si>
+    <t>AKSHAY1996</t>
+  </si>
+  <si>
+    <t>1996-11-26</t>
+  </si>
+  <si>
+    <t>26/11/1996</t>
+  </si>
+  <si>
+    <t>AMRS1234</t>
+  </si>
+  <si>
+    <t>1971-05-10</t>
+  </si>
+  <si>
+    <t>10/05/1971</t>
+  </si>
+  <si>
+    <t>AVCO0422</t>
+  </si>
+  <si>
+    <t>1999-01-29</t>
+  </si>
+  <si>
+    <t>29/01/1999</t>
+  </si>
+  <si>
+    <t>BANB1242</t>
+  </si>
+  <si>
+    <t>2000-04-04</t>
+  </si>
+  <si>
+    <t>04/04/2000</t>
+  </si>
+  <si>
+    <t>BANB1244</t>
+  </si>
+  <si>
+    <t>1952-06-01</t>
+  </si>
+  <si>
+    <t>01/06/1952</t>
+  </si>
+  <si>
+    <t>BRD1117</t>
+  </si>
+  <si>
+    <t>1967-07-28</t>
+  </si>
+  <si>
+    <t>28/07/1967</t>
+  </si>
+  <si>
+    <t>BRD1187</t>
+  </si>
+  <si>
+    <t>1966-11-17</t>
+  </si>
+  <si>
+    <t>17/11/1966</t>
+  </si>
+  <si>
+    <t>BRD1191</t>
+  </si>
+  <si>
+    <t>1987-03-09</t>
+  </si>
+  <si>
+    <t>09/03/1987</t>
+  </si>
+  <si>
+    <t>BRD1192</t>
+  </si>
+  <si>
+    <t>1982-06-02</t>
+  </si>
+  <si>
+    <t>02/06/1982</t>
+  </si>
+  <si>
+    <t>BRD1194</t>
+  </si>
+  <si>
+    <t>1937-09-05</t>
+  </si>
+  <si>
+    <t>05/09/1937</t>
+  </si>
+  <si>
+    <t>BRD1207</t>
+  </si>
+  <si>
+    <t>1985-06-17</t>
+  </si>
+  <si>
+    <t>17/06/1985</t>
+  </si>
+  <si>
+    <t>BRD1209</t>
+  </si>
+  <si>
+    <t>1962-12-14</t>
+  </si>
+  <si>
+    <t>14/12/1962</t>
+  </si>
+  <si>
+    <t>BRD1210</t>
+  </si>
+  <si>
+    <t>1995-08-11</t>
+  </si>
+  <si>
+    <t>11/08/1995</t>
+  </si>
+  <si>
+    <t>BRD1217</t>
+  </si>
+  <si>
+    <t>1952-01-30</t>
+  </si>
+  <si>
+    <t>30/01/1952</t>
+  </si>
+  <si>
+    <t>BRD1220</t>
+  </si>
+  <si>
+    <t>1982-07-01</t>
+  </si>
+  <si>
+    <t>01/07/1982</t>
+  </si>
+  <si>
+    <t>BRD1222</t>
+  </si>
+  <si>
+    <t>1983-10-06</t>
+  </si>
+  <si>
+    <t>06/10/1983</t>
+  </si>
+  <si>
+    <t>BRD1223</t>
+  </si>
+  <si>
+    <t>1960-03-10</t>
+  </si>
+  <si>
+    <t>10/03/1960</t>
+  </si>
+  <si>
+    <t>BRD1229</t>
+  </si>
+  <si>
+    <t>1991-01-24</t>
+  </si>
+  <si>
+    <t>24/01/1991</t>
+  </si>
+  <si>
+    <t>BRD1261</t>
+  </si>
+  <si>
+    <t>1970-05-13</t>
+  </si>
+  <si>
+    <t>13/05/1970</t>
+  </si>
+  <si>
+    <t>BRD1281</t>
+  </si>
+  <si>
+    <t>1975-03-01</t>
+  </si>
+  <si>
+    <t>01/03/1975</t>
+  </si>
+  <si>
+    <t>BRD2673</t>
+  </si>
+  <si>
+    <t>1995-07-16</t>
+  </si>
+  <si>
+    <t>16/07/1995</t>
+  </si>
+  <si>
+    <t>BRD695</t>
+  </si>
+  <si>
+    <t>1964-10-19</t>
+  </si>
+  <si>
+    <t>19/10/1964</t>
+  </si>
+  <si>
+    <t>BRD948</t>
+  </si>
+  <si>
+    <t>1969-06-16</t>
+  </si>
+  <si>
+    <t>16/06/1969</t>
+  </si>
+  <si>
+    <t>CPPUNE51</t>
+  </si>
+  <si>
+    <t>1974-05-28</t>
+  </si>
+  <si>
+    <t>28/05/1974</t>
+  </si>
+  <si>
+    <t>DL35491</t>
+  </si>
+  <si>
+    <t>1967-11-10</t>
+  </si>
+  <si>
+    <t>10/11/1967</t>
+  </si>
+  <si>
+    <t>DPML1223</t>
+  </si>
+  <si>
+    <t>2002-06-13</t>
+  </si>
+  <si>
+    <t>13/06/2002</t>
+  </si>
+  <si>
+    <t>DRMW1249</t>
+  </si>
+  <si>
+    <t>1994-05-22</t>
+  </si>
+  <si>
+    <t>22/05/1994</t>
+  </si>
+  <si>
+    <t>DSTC0024</t>
+  </si>
+  <si>
+    <t>1990-02-28</t>
+  </si>
+  <si>
+    <t>28/02/1990</t>
+  </si>
+  <si>
+    <t>EAOPE36178</t>
+  </si>
+  <si>
+    <t>1995-12-30</t>
+  </si>
+  <si>
+    <t>30/12/1995</t>
+  </si>
+  <si>
+    <t>EAS467</t>
+  </si>
+  <si>
+    <t>1957-08-01</t>
+  </si>
+  <si>
+    <t>01/08/1957</t>
+  </si>
+  <si>
+    <t>EAS468</t>
+  </si>
+  <si>
+    <t>1990-04-10</t>
+  </si>
+  <si>
+    <t>10/04/1990</t>
+  </si>
+  <si>
+    <t>EAS469</t>
+  </si>
+  <si>
+    <t>1968-03-08</t>
+  </si>
+  <si>
+    <t>08/03/1968</t>
+  </si>
+  <si>
+    <t>EHYD633800</t>
+  </si>
+  <si>
+    <t>1992-04-09</t>
+  </si>
+  <si>
+    <t>09/04/1992</t>
+  </si>
+  <si>
+    <t>H22152</t>
+  </si>
+  <si>
+    <t>1995-01-01</t>
+  </si>
+  <si>
+    <t>01/01/1995</t>
+  </si>
+  <si>
+    <t>JASH115</t>
+  </si>
+  <si>
+    <t>1969-12-24</t>
+  </si>
+  <si>
+    <t>24/12/1969</t>
+  </si>
+  <si>
+    <t>JASH122</t>
+  </si>
+  <si>
+    <t>1971-07-07</t>
+  </si>
+  <si>
+    <t>07/07/1971</t>
+  </si>
+  <si>
+    <t>JASH123</t>
+  </si>
+  <si>
+    <t>1989-03-19</t>
+  </si>
+  <si>
+    <t>19/03/1989</t>
+  </si>
+  <si>
+    <t>JASH125</t>
+  </si>
+  <si>
+    <t>1995-04-25</t>
+  </si>
+  <si>
+    <t>25/04/1995</t>
+  </si>
+  <si>
+    <t>JASH126</t>
+  </si>
+  <si>
+    <t>1988-01-09</t>
+  </si>
+  <si>
+    <t>09/01/1988</t>
+  </si>
+  <si>
+    <t>JASH128</t>
+  </si>
+  <si>
+    <t>1990-08-11</t>
+  </si>
+  <si>
+    <t>11/08/1990</t>
+  </si>
+  <si>
+    <t>JASH133</t>
+  </si>
+  <si>
+    <t>1989-03-26</t>
+  </si>
+  <si>
+    <t>26/03/1989</t>
+  </si>
+  <si>
+    <t>KARTICK79</t>
+  </si>
+  <si>
+    <t>1979-01-15</t>
+  </si>
+  <si>
+    <t>15/01/1979</t>
+  </si>
+  <si>
+    <t>KNIS1971</t>
+  </si>
+  <si>
+    <t>1971-06-01</t>
+  </si>
+  <si>
+    <t>01/06/1971</t>
+  </si>
+  <si>
+    <t>MARC1000</t>
+  </si>
+  <si>
+    <t>1989-12-21</t>
+  </si>
+  <si>
+    <t>21/12/1989</t>
+  </si>
+  <si>
+    <t>MARC1001</t>
+  </si>
+  <si>
+    <t>1983-02-14</t>
+  </si>
+  <si>
+    <t>14/02/1983</t>
+  </si>
+  <si>
+    <t>MARC1003</t>
+  </si>
+  <si>
+    <t>1980-06-08</t>
+  </si>
+  <si>
+    <t>08/06/1980</t>
+  </si>
+  <si>
+    <t>MARC1004</t>
+  </si>
+  <si>
+    <t>1970-08-23</t>
+  </si>
+  <si>
+    <t>23/08/1970</t>
+  </si>
+  <si>
+    <t>MARC1031</t>
+  </si>
+  <si>
+    <t>1991-06-06</t>
+  </si>
+  <si>
+    <t>06/06/1991</t>
+  </si>
+  <si>
+    <t>MARC3229</t>
+  </si>
+  <si>
+    <t>1967-12-10</t>
+  </si>
+  <si>
+    <t>10/12/1967</t>
+  </si>
+  <si>
+    <t>MARC3232</t>
+  </si>
+  <si>
+    <t>1949-07-07</t>
+  </si>
+  <si>
+    <t>07/07/1949</t>
+  </si>
+  <si>
+    <t>MARC3240</t>
+  </si>
+  <si>
+    <t>1975-03-20</t>
+  </si>
+  <si>
+    <t>20/03/1975</t>
+  </si>
+  <si>
+    <t>MOSTI1579</t>
+  </si>
+  <si>
+    <t>1984-03-05</t>
+  </si>
+  <si>
+    <t>05/03/1984</t>
+  </si>
+  <si>
+    <t>MTMFDVG001</t>
+  </si>
+  <si>
+    <t>1985-05-10</t>
+  </si>
+  <si>
+    <t>10/05/1985</t>
+  </si>
+  <si>
+    <t>NAGD460</t>
+  </si>
+  <si>
+    <t>1959-12-22</t>
+  </si>
+  <si>
+    <t>22/12/1959</t>
+  </si>
+  <si>
+    <t>NAGD495</t>
+  </si>
+  <si>
+    <t>1964-01-09</t>
+  </si>
+  <si>
+    <t>09/01/1964</t>
+  </si>
+  <si>
+    <t>NPUP1466</t>
+  </si>
+  <si>
+    <t>1999-10-13</t>
+  </si>
+  <si>
+    <t>13/10/1999</t>
+  </si>
+  <si>
+    <t>NPUP1472</t>
+  </si>
+  <si>
+    <t>1969-04-01</t>
+  </si>
+  <si>
+    <t>01/04/1969</t>
+  </si>
+  <si>
+    <t>NPUP1476</t>
+  </si>
+  <si>
+    <t>1978-06-25</t>
+  </si>
+  <si>
+    <t>25/06/1978</t>
+  </si>
+  <si>
+    <t>OMJA1160</t>
+  </si>
+  <si>
+    <t>1976-04-13</t>
+  </si>
+  <si>
+    <t>13/04/1976</t>
+  </si>
+  <si>
+    <t>OMRJ1839</t>
+  </si>
+  <si>
+    <t>1986-07-23</t>
+  </si>
+  <si>
+    <t>23/07/1986</t>
+  </si>
+  <si>
+    <t>RETK2909</t>
+  </si>
+  <si>
+    <t>1973-12-21</t>
+  </si>
+  <si>
+    <t>21/12/1973</t>
+  </si>
+  <si>
+    <t>RETK2910</t>
+  </si>
+  <si>
+    <t>1986-05-05</t>
+  </si>
+  <si>
+    <t>05/05/1986</t>
+  </si>
+  <si>
+    <t>RETK2914</t>
+  </si>
+  <si>
+    <t>1950-02-02</t>
+  </si>
+  <si>
+    <t>02/02/1950</t>
+  </si>
+  <si>
+    <t>RETK2917</t>
+  </si>
+  <si>
+    <t>1997-08-28</t>
+  </si>
+  <si>
+    <t>28/08/1997</t>
+  </si>
+  <si>
+    <t>RETK2919</t>
+  </si>
+  <si>
+    <t>1956-11-11</t>
+  </si>
+  <si>
+    <t>11/11/1956</t>
+  </si>
+  <si>
+    <t>RETK2922</t>
+  </si>
+  <si>
+    <t>1954-01-03</t>
+  </si>
+  <si>
+    <t>03/01/1954</t>
+  </si>
+  <si>
+    <t>RETK2923</t>
+  </si>
+  <si>
+    <t>1985-04-27</t>
+  </si>
+  <si>
+    <t>27/04/1985</t>
+  </si>
+  <si>
+    <t>RETK2924</t>
+  </si>
+  <si>
+    <t>2000-06-17</t>
+  </si>
+  <si>
+    <t>17/06/2000</t>
+  </si>
+  <si>
+    <t>RETK2925</t>
+  </si>
+  <si>
+    <t>1969-10-31</t>
+  </si>
+  <si>
+    <t>31/10/1969</t>
+  </si>
+  <si>
+    <t>RETK2927</t>
+  </si>
+  <si>
+    <t>1962-03-14</t>
+  </si>
+  <si>
+    <t>14/03/1962</t>
+  </si>
+  <si>
+    <t>RETK2929</t>
+  </si>
+  <si>
+    <t>1989-06-25</t>
+  </si>
+  <si>
+    <t>25/06/1989</t>
+  </si>
+  <si>
+    <t>RETK2930</t>
+  </si>
+  <si>
+    <t>1987-11-26</t>
+  </si>
+  <si>
+    <t>26/11/1987</t>
+  </si>
+  <si>
+    <t>RETK2931</t>
+  </si>
+  <si>
+    <t>1979-10-07</t>
+  </si>
+  <si>
+    <t>07/10/1979</t>
+  </si>
+  <si>
+    <t>RETK2932</t>
+  </si>
+  <si>
+    <t>1979-10-08</t>
+  </si>
+  <si>
+    <t>08/10/1979</t>
+  </si>
+  <si>
+    <t>RETK2933</t>
+  </si>
+  <si>
+    <t>1989-05-03</t>
+  </si>
+  <si>
+    <t>03/05/1989</t>
+  </si>
+  <si>
+    <t>RETK2934</t>
+  </si>
+  <si>
+    <t>1995-04-29</t>
+  </si>
+  <si>
+    <t>29/04/1995</t>
+  </si>
+  <si>
+    <t>RETK2936</t>
+  </si>
+  <si>
+    <t>1989-08-12</t>
+  </si>
+  <si>
+    <t>12/08/1989</t>
+  </si>
+  <si>
+    <t>RETK2937</t>
+  </si>
+  <si>
+    <t>RETK2938</t>
+  </si>
+  <si>
+    <t>1997-10-24</t>
+  </si>
+  <si>
+    <t>24/10/1997</t>
+  </si>
+  <si>
+    <t>RETK2940</t>
+  </si>
+  <si>
+    <t>1991-07-17</t>
+  </si>
+  <si>
+    <t>17/07/1991</t>
+  </si>
+  <si>
+    <t>RETK2941</t>
+  </si>
+  <si>
+    <t>1964-12-31</t>
+  </si>
+  <si>
+    <t>31/12/1964</t>
+  </si>
+  <si>
+    <t>RETK2942</t>
+  </si>
+  <si>
+    <t>1994-02-26</t>
+  </si>
+  <si>
+    <t>26/02/1994</t>
+  </si>
+  <si>
+    <t>RETK2943</t>
+  </si>
+  <si>
+    <t>1983-01-01</t>
+  </si>
+  <si>
+    <t>01/01/1983</t>
+  </si>
+  <si>
+    <t>RETK2944</t>
+  </si>
+  <si>
+    <t>1987-10-10</t>
+  </si>
+  <si>
+    <t>10/10/1987</t>
+  </si>
+  <si>
+    <t>RETK2945</t>
+  </si>
+  <si>
+    <t>1961-01-02</t>
+  </si>
+  <si>
+    <t>02/01/1961</t>
+  </si>
+  <si>
+    <t>RETK2946</t>
+  </si>
+  <si>
+    <t>1990-06-01</t>
+  </si>
+  <si>
+    <t>01/06/1990</t>
+  </si>
+  <si>
+    <t>RETK2948</t>
+  </si>
+  <si>
+    <t>1971-05-01</t>
+  </si>
+  <si>
+    <t>01/05/1971</t>
+  </si>
+  <si>
+    <t>RETK2949</t>
+  </si>
+  <si>
+    <t>1964-03-05</t>
+  </si>
+  <si>
+    <t>05/03/1964</t>
+  </si>
+  <si>
+    <t>RETK2950</t>
+  </si>
+  <si>
+    <t>1995-04-27</t>
+  </si>
+  <si>
+    <t>27/04/1995</t>
+  </si>
+  <si>
+    <t>RETK2951</t>
+  </si>
+  <si>
+    <t>1962-08-14</t>
+  </si>
+  <si>
+    <t>14/08/1962</t>
+  </si>
+  <si>
+    <t>RETK2952</t>
+  </si>
+  <si>
+    <t>1993-11-23</t>
+  </si>
+  <si>
+    <t>23/11/1993</t>
+  </si>
+  <si>
+    <t>RETK2954</t>
+  </si>
+  <si>
+    <t>1985-05-04</t>
+  </si>
+  <si>
+    <t>04/05/1985</t>
+  </si>
+  <si>
+    <t>RETK2956</t>
+  </si>
+  <si>
+    <t>1970-02-04</t>
+  </si>
+  <si>
+    <t>04/02/1970</t>
+  </si>
+  <si>
+    <t>RETK2957</t>
+  </si>
+  <si>
+    <t>1979-03-03</t>
+  </si>
+  <si>
+    <t>03/03/1979</t>
+  </si>
+  <si>
+    <t>RETK2958</t>
+  </si>
+  <si>
+    <t>1992-12-21</t>
+  </si>
+  <si>
+    <t>21/12/1992</t>
+  </si>
+  <si>
+    <t>RETK2960</t>
+  </si>
+  <si>
+    <t>1982-06-09</t>
+  </si>
+  <si>
+    <t>09/06/1982</t>
+  </si>
+  <si>
+    <t>RETK2964</t>
+  </si>
+  <si>
+    <t>1981-09-06</t>
+  </si>
+  <si>
+    <t>06/09/1981</t>
+  </si>
+  <si>
+    <t>RETK2965</t>
+  </si>
+  <si>
+    <t>1967-07-30</t>
+  </si>
+  <si>
+    <t>30/07/1967</t>
+  </si>
+  <si>
+    <t>RETK2967</t>
+  </si>
+  <si>
+    <t>1994-08-18</t>
+  </si>
+  <si>
+    <t>18/08/1994</t>
+  </si>
+  <si>
+    <t>RETK2968</t>
+  </si>
+  <si>
+    <t>1984-11-30</t>
+  </si>
+  <si>
+    <t>30/11/1984</t>
+  </si>
+  <si>
+    <t>RETK2970</t>
+  </si>
+  <si>
+    <t>1949-09-03</t>
+  </si>
+  <si>
+    <t>03/09/1949</t>
+  </si>
+  <si>
+    <t>RETK2971</t>
+  </si>
+  <si>
+    <t>1986-02-02</t>
+  </si>
+  <si>
+    <t>02/02/1986</t>
+  </si>
+  <si>
+    <t>RETK2972</t>
+  </si>
+  <si>
+    <t>1983-12-24</t>
+  </si>
+  <si>
+    <t>24/12/1983</t>
+  </si>
+  <si>
+    <t>RETK2973</t>
+  </si>
+  <si>
+    <t>1963-06-02</t>
+  </si>
+  <si>
+    <t>02/06/1963</t>
+  </si>
+  <si>
+    <t>RETK2974</t>
+  </si>
+  <si>
+    <t>1979-08-15</t>
+  </si>
+  <si>
+    <t>15/08/1979</t>
+  </si>
+  <si>
+    <t>RETK2976</t>
+  </si>
+  <si>
+    <t>1993-03-26</t>
+  </si>
+  <si>
+    <t>26/03/1993</t>
+  </si>
+  <si>
+    <t>RETK2977</t>
+  </si>
+  <si>
+    <t>1978-01-03</t>
+  </si>
+  <si>
+    <t>03/01/1978</t>
+  </si>
+  <si>
+    <t>RETK2979</t>
+  </si>
+  <si>
+    <t>1942-02-08</t>
+  </si>
+  <si>
+    <t>08/02/1942</t>
+  </si>
+  <si>
+    <t>RETK2982</t>
+  </si>
+  <si>
+    <t>1993-03-05</t>
+  </si>
+  <si>
+    <t>05/03/1993</t>
+  </si>
+  <si>
+    <t>RETK2983</t>
+  </si>
+  <si>
+    <t>1999-06-16</t>
+  </si>
+  <si>
+    <t>16/06/1999</t>
+  </si>
+  <si>
+    <t>RETK2984</t>
+  </si>
+  <si>
+    <t>1992-09-08</t>
+  </si>
+  <si>
+    <t>08/09/1992</t>
+  </si>
+  <si>
+    <t>RETK2985</t>
+  </si>
+  <si>
+    <t>1978-01-02</t>
+  </si>
+  <si>
+    <t>02/01/1978</t>
+  </si>
+  <si>
+    <t>RETK2987</t>
+  </si>
+  <si>
+    <t>1990-12-28</t>
+  </si>
+  <si>
+    <t>28/12/1990</t>
+  </si>
+  <si>
+    <t>RETK2988</t>
+  </si>
+  <si>
+    <t>1991-12-18</t>
+  </si>
+  <si>
+    <t>18/12/1991</t>
+  </si>
+  <si>
+    <t>RETK2989</t>
+  </si>
+  <si>
+    <t>1989-11-16</t>
+  </si>
+  <si>
+    <t>16/11/1989</t>
+  </si>
+  <si>
+    <t>RETK2990</t>
+  </si>
+  <si>
+    <t>1997-01-23</t>
+  </si>
+  <si>
+    <t>23/01/1997</t>
+  </si>
+  <si>
+    <t>RETK2992</t>
+  </si>
+  <si>
+    <t>1959-12-28</t>
+  </si>
+  <si>
+    <t>28/12/1959</t>
+  </si>
+  <si>
+    <t>RETK2993</t>
+  </si>
+  <si>
+    <t>1958-02-04</t>
+  </si>
+  <si>
+    <t>04/02/1958</t>
+  </si>
+  <si>
+    <t>RETK2996</t>
+  </si>
+  <si>
+    <t>1956-05-11</t>
+  </si>
+  <si>
+    <t>11/05/1956</t>
+  </si>
+  <si>
+    <t>RETK2997</t>
+  </si>
+  <si>
+    <t>1980-11-15</t>
+  </si>
+  <si>
+    <t>15/11/1980</t>
+  </si>
+  <si>
+    <t>RETK3000</t>
+  </si>
+  <si>
+    <t>1987-10-30</t>
+  </si>
+  <si>
+    <t>30/10/1987</t>
+  </si>
+  <si>
+    <t>RETK3001</t>
+  </si>
+  <si>
+    <t>1983-03-15</t>
+  </si>
+  <si>
+    <t>15/03/1983</t>
+  </si>
+  <si>
+    <t>RETK3002</t>
+  </si>
+  <si>
+    <t>1973-01-01</t>
+  </si>
+  <si>
+    <t>01/01/1973</t>
+  </si>
+  <si>
+    <t>RETK3003</t>
+  </si>
+  <si>
+    <t>1974-08-30</t>
+  </si>
+  <si>
+    <t>30/08/1974</t>
+  </si>
+  <si>
+    <t>RETK3004</t>
+  </si>
+  <si>
+    <t>1989-06-19</t>
+  </si>
+  <si>
+    <t>19/06/1989</t>
+  </si>
+  <si>
+    <t>RETK3006</t>
+  </si>
+  <si>
+    <t>1987-06-07</t>
+  </si>
+  <si>
+    <t>07/06/1987</t>
+  </si>
+  <si>
+    <t>RETK3007</t>
+  </si>
+  <si>
+    <t>1984-05-08</t>
+  </si>
+  <si>
+    <t>08/05/1984</t>
+  </si>
+  <si>
+    <t>RETK3008</t>
+  </si>
+  <si>
+    <t>1984-02-24</t>
+  </si>
+  <si>
+    <t>24/02/1984</t>
+  </si>
+  <si>
+    <t>RETK3010</t>
+  </si>
+  <si>
+    <t>1965-01-08</t>
+  </si>
+  <si>
+    <t>08/01/1965</t>
+  </si>
+  <si>
+    <t>RETK3012</t>
+  </si>
+  <si>
+    <t>1972-12-01</t>
+  </si>
+  <si>
+    <t>01/12/1972</t>
+  </si>
+  <si>
+    <t>RETK3013</t>
+  </si>
+  <si>
+    <t>1983-05-14</t>
+  </si>
+  <si>
+    <t>14/05/1983</t>
+  </si>
+  <si>
+    <t>RETK3014</t>
+  </si>
+  <si>
+    <t>1951-01-16</t>
+  </si>
+  <si>
+    <t>16/01/1951</t>
+  </si>
+  <si>
+    <t>RETK3015</t>
+  </si>
+  <si>
+    <t>1967-02-08</t>
+  </si>
+  <si>
+    <t>08/02/1967</t>
+  </si>
+  <si>
+    <t>RETK3016</t>
+  </si>
+  <si>
+    <t>1970-01-23</t>
+  </si>
+  <si>
+    <t>23/01/1970</t>
+  </si>
+  <si>
+    <t>RETK3017</t>
+  </si>
+  <si>
+    <t>1994-03-26</t>
+  </si>
+  <si>
+    <t>26/03/1994</t>
+  </si>
+  <si>
+    <t>RETK3019</t>
+  </si>
+  <si>
+    <t>1992-02-07</t>
+  </si>
+  <si>
+    <t>07/02/1992</t>
+  </si>
+  <si>
+    <t>RETK3020</t>
+  </si>
+  <si>
+    <t>1958-10-19</t>
+  </si>
+  <si>
+    <t>19/10/1958</t>
+  </si>
+  <si>
+    <t>RETK3021</t>
+  </si>
+  <si>
+    <t>1989-09-04</t>
+  </si>
+  <si>
+    <t>04/09/1989</t>
+  </si>
+  <si>
+    <t>RETK3023</t>
+  </si>
+  <si>
+    <t>1985-03-18</t>
+  </si>
+  <si>
+    <t>18/03/1985</t>
+  </si>
+  <si>
+    <t>RETK3025</t>
+  </si>
+  <si>
+    <t>1990-07-09</t>
+  </si>
+  <si>
+    <t>09/07/1990</t>
+  </si>
+  <si>
+    <t>RETK3029</t>
+  </si>
+  <si>
+    <t>1995-06-03</t>
+  </si>
+  <si>
+    <t>03/06/1995</t>
+  </si>
+  <si>
+    <t>RETK3031</t>
+  </si>
+  <si>
+    <t>1979-10-01</t>
+  </si>
+  <si>
+    <t>01/10/1979</t>
+  </si>
+  <si>
+    <t>RETK3032</t>
+  </si>
+  <si>
+    <t>1985-06-06</t>
+  </si>
+  <si>
+    <t>06/06/1985</t>
+  </si>
+  <si>
+    <t>RETK3033</t>
+  </si>
+  <si>
+    <t>1971-02-01</t>
+  </si>
+  <si>
+    <t>01/02/1971</t>
+  </si>
+  <si>
+    <t>RETK3034</t>
+  </si>
+  <si>
+    <t>1983-12-16</t>
+  </si>
+  <si>
+    <t>16/12/1983</t>
+  </si>
+  <si>
+    <t>RETK3036</t>
+  </si>
+  <si>
+    <t>1988-04-15</t>
+  </si>
+  <si>
+    <t>15/04/1988</t>
+  </si>
+  <si>
+    <t>RETK3037</t>
+  </si>
+  <si>
+    <t>1984-02-21</t>
+  </si>
+  <si>
+    <t>21/02/1984</t>
+  </si>
+  <si>
+    <t>RETK3038</t>
+  </si>
+  <si>
+    <t>1986-02-22</t>
+  </si>
+  <si>
+    <t>22/02/1986</t>
+  </si>
+  <si>
+    <t>RETK3039</t>
+  </si>
+  <si>
+    <t>1995-08-27</t>
+  </si>
+  <si>
+    <t>27/08/1995</t>
+  </si>
+  <si>
+    <t>RETK3040</t>
+  </si>
+  <si>
+    <t>1989-05-10</t>
+  </si>
+  <si>
+    <t>10/05/1989</t>
+  </si>
+  <si>
+    <t>RETK3041</t>
+  </si>
+  <si>
+    <t>1991-04-20</t>
+  </si>
+  <si>
+    <t>20/04/1991</t>
+  </si>
+  <si>
+    <t>RETK3042</t>
+  </si>
+  <si>
+    <t>1972-09-21</t>
+  </si>
+  <si>
+    <t>21/09/1972</t>
+  </si>
+  <si>
+    <t>RETK3044</t>
+  </si>
+  <si>
+    <t>1985-05-15</t>
+  </si>
+  <si>
+    <t>15/05/1985</t>
+  </si>
+  <si>
+    <t>RETK3046</t>
+  </si>
+  <si>
+    <t>1992-05-29</t>
+  </si>
+  <si>
+    <t>29/05/1992</t>
+  </si>
+  <si>
+    <t>RETK3047</t>
+  </si>
+  <si>
+    <t>1964-01-01</t>
+  </si>
+  <si>
+    <t>01/01/1964</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <numFmts count="0"/>
+  <fonts count="25" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -219,6 +1654,121 @@
       <color theme="1"/>
       <name val="Consolas"/>
       <family val="3"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
     </font>
   </fonts>
   <fills count="2">
@@ -241,7 +1791,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -249,6 +1799,29 @@
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="true"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -532,9 +2105,9 @@
   <dimension ref="A1:B23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="34.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="51.5703125" style="1" customWidth="1"/>
-    <col min="3" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="1" width="34.7109375"/>
+    <col min="2" max="2" customWidth="true" style="1" width="51.5703125"/>
+    <col min="3" max="16384" style="1" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -732,91 +2305,91 @@
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="28" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="9.42578125"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="16.28515625"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="10.85546875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="12.42578125"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="28.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="13.85546875"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="14.7109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="9.85546875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+      <c r="A1" t="s" s="0">
         <v>44</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" t="s" s="0">
         <v>45</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" t="s" s="0">
         <v>46</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" t="s" s="0">
         <v>47</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" t="s" s="0">
         <v>48</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" t="s" s="0">
         <v>49</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" t="s" s="0">
         <v>50</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" t="s" s="0">
         <v>51</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2">
+      <c r="A2" s="0">
         <v>28135</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>52</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" t="s" s="0">
         <v>57</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" t="s" s="0">
         <v>7</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" t="s" s="0">
         <v>5</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" t="s" s="0">
         <v>53</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" t="s" s="0">
         <v>9</v>
       </c>
-      <c r="H2">
+      <c r="H2" s="0">
         <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3">
+      <c r="A3" s="0">
         <v>40445</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" t="s" s="0">
         <v>56</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" t="s" s="0">
         <v>58</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" t="s" s="0">
         <v>54</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" t="s" s="0">
         <v>55</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F3" t="s" s="0">
         <v>53</v>
       </c>
-      <c r="G3" t="s">
+      <c r="G3" t="s" s="0">
         <v>59</v>
       </c>
-      <c r="H3">
+      <c r="H3" s="0">
         <v>1</v>
       </c>
     </row>
@@ -824,4 +2397,888 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:E51"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <cols>
+    <col min="1" max="1" width="9.85546875" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="10.13671875" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="13.296875" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="9.66015625" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="9.6484375" customWidth="true" bestFit="true"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="25">
+        <v>46</v>
+      </c>
+      <c r="B1" t="s" s="25">
+        <v>60</v>
+      </c>
+      <c r="C1" t="s" s="25">
+        <v>61</v>
+      </c>
+      <c r="D1" t="s" s="25">
+        <v>62</v>
+      </c>
+      <c r="E1" t="s" s="25">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>256</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>257</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>258</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="E2" t="s" s="0">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>259</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>260</v>
+      </c>
+      <c r="C3" t="s" s="0">
+        <v>261</v>
+      </c>
+      <c r="D3" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="E3" t="s" s="0">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>262</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>263</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>264</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="E4" t="s" s="0">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>265</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>266</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>267</v>
+      </c>
+      <c r="D5" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="E5" t="s" s="0">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>268</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>269</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>270</v>
+      </c>
+      <c r="D6" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="E6" t="s" s="0">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>271</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>272</v>
+      </c>
+      <c r="C7" t="s" s="0">
+        <v>273</v>
+      </c>
+      <c r="D7" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="E7" t="s" s="0">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="0">
+        <v>274</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>275</v>
+      </c>
+      <c r="C8" t="s" s="0">
+        <v>276</v>
+      </c>
+      <c r="D8" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="E8" t="s" s="0">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="0">
+        <v>277</v>
+      </c>
+      <c r="B9" t="s" s="0">
+        <v>278</v>
+      </c>
+      <c r="C9" t="s" s="0">
+        <v>279</v>
+      </c>
+      <c r="D9" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="E9" t="s" s="0">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s" s="0">
+        <v>280</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>281</v>
+      </c>
+      <c r="C10" t="s" s="0">
+        <v>282</v>
+      </c>
+      <c r="D10" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="E10" t="s" s="0">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s" s="0">
+        <v>283</v>
+      </c>
+      <c r="B11" t="s" s="0">
+        <v>284</v>
+      </c>
+      <c r="C11" t="s" s="0">
+        <v>285</v>
+      </c>
+      <c r="D11" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="E11" t="s" s="0">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s" s="0">
+        <v>286</v>
+      </c>
+      <c r="B12" t="s" s="0">
+        <v>287</v>
+      </c>
+      <c r="C12" t="s" s="0">
+        <v>288</v>
+      </c>
+      <c r="D12" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="E12" t="s" s="0">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s" s="0">
+        <v>289</v>
+      </c>
+      <c r="B13" t="s" s="0">
+        <v>290</v>
+      </c>
+      <c r="C13" t="s" s="0">
+        <v>291</v>
+      </c>
+      <c r="D13" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="E13" t="s" s="0">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s" s="0">
+        <v>292</v>
+      </c>
+      <c r="B14" t="s" s="0">
+        <v>293</v>
+      </c>
+      <c r="C14" t="s" s="0">
+        <v>294</v>
+      </c>
+      <c r="D14" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="E14" t="s" s="0">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s" s="0">
+        <v>295</v>
+      </c>
+      <c r="B15" t="s" s="0">
+        <v>296</v>
+      </c>
+      <c r="C15" t="s" s="0">
+        <v>297</v>
+      </c>
+      <c r="D15" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="E15" t="s" s="0">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s" s="0">
+        <v>298</v>
+      </c>
+      <c r="B16" t="s" s="0">
+        <v>299</v>
+      </c>
+      <c r="C16" t="s" s="0">
+        <v>300</v>
+      </c>
+      <c r="D16" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="E16" t="s" s="0">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s" s="0">
+        <v>301</v>
+      </c>
+      <c r="B17" t="s" s="0">
+        <v>302</v>
+      </c>
+      <c r="C17" t="s" s="0">
+        <v>303</v>
+      </c>
+      <c r="D17" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="E17" t="s" s="0">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s" s="0">
+        <v>304</v>
+      </c>
+      <c r="B18" t="s" s="0">
+        <v>305</v>
+      </c>
+      <c r="C18" t="s" s="0">
+        <v>306</v>
+      </c>
+      <c r="D18" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="E18" t="s" s="0">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s" s="0">
+        <v>307</v>
+      </c>
+      <c r="B19" t="s" s="0">
+        <v>302</v>
+      </c>
+      <c r="C19" t="s" s="0">
+        <v>303</v>
+      </c>
+      <c r="D19" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="E19" t="s" s="0">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s" s="0">
+        <v>308</v>
+      </c>
+      <c r="B20" t="s" s="0">
+        <v>309</v>
+      </c>
+      <c r="C20" t="s" s="0">
+        <v>310</v>
+      </c>
+      <c r="D20" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="E20" t="s" s="0">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s" s="0">
+        <v>311</v>
+      </c>
+      <c r="B21" t="s" s="0">
+        <v>312</v>
+      </c>
+      <c r="C21" t="s" s="0">
+        <v>313</v>
+      </c>
+      <c r="D21" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="E21" t="s" s="0">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s" s="0">
+        <v>314</v>
+      </c>
+      <c r="B22" t="s" s="0">
+        <v>315</v>
+      </c>
+      <c r="C22" t="s" s="0">
+        <v>316</v>
+      </c>
+      <c r="D22" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="E22" t="s" s="0">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s" s="0">
+        <v>317</v>
+      </c>
+      <c r="B23" t="s" s="0">
+        <v>318</v>
+      </c>
+      <c r="C23" t="s" s="0">
+        <v>319</v>
+      </c>
+      <c r="D23" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="E23" t="s" s="0">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="s" s="0">
+        <v>320</v>
+      </c>
+      <c r="B24" t="s" s="0">
+        <v>321</v>
+      </c>
+      <c r="C24" t="s" s="0">
+        <v>322</v>
+      </c>
+      <c r="D24" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="E24" t="s" s="0">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="s" s="0">
+        <v>323</v>
+      </c>
+      <c r="B25" t="s" s="0">
+        <v>324</v>
+      </c>
+      <c r="C25" t="s" s="0">
+        <v>325</v>
+      </c>
+      <c r="D25" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="E25" t="s" s="0">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="s" s="0">
+        <v>326</v>
+      </c>
+      <c r="B26" t="s" s="0">
+        <v>327</v>
+      </c>
+      <c r="C26" t="s" s="0">
+        <v>328</v>
+      </c>
+      <c r="D26" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="E26" t="s" s="0">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="s" s="0">
+        <v>329</v>
+      </c>
+      <c r="B27" t="s" s="0">
+        <v>330</v>
+      </c>
+      <c r="C27" t="s" s="0">
+        <v>331</v>
+      </c>
+      <c r="D27" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="E27" t="s" s="0">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="s" s="0">
+        <v>332</v>
+      </c>
+      <c r="B28" t="s" s="0">
+        <v>333</v>
+      </c>
+      <c r="C28" t="s" s="0">
+        <v>334</v>
+      </c>
+      <c r="D28" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="E28" t="s" s="0">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="s" s="0">
+        <v>335</v>
+      </c>
+      <c r="B29" t="s" s="0">
+        <v>336</v>
+      </c>
+      <c r="C29" t="s" s="0">
+        <v>337</v>
+      </c>
+      <c r="D29" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="E29" t="s" s="0">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="s" s="0">
+        <v>338</v>
+      </c>
+      <c r="B30" t="s" s="0">
+        <v>339</v>
+      </c>
+      <c r="C30" t="s" s="0">
+        <v>340</v>
+      </c>
+      <c r="D30" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="E30" t="s" s="0">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="s" s="0">
+        <v>341</v>
+      </c>
+      <c r="B31" t="s" s="0">
+        <v>342</v>
+      </c>
+      <c r="C31" t="s" s="0">
+        <v>343</v>
+      </c>
+      <c r="D31" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="E31" t="s" s="0">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="s" s="0">
+        <v>344</v>
+      </c>
+      <c r="B32" t="s" s="0">
+        <v>345</v>
+      </c>
+      <c r="C32" t="s" s="0">
+        <v>346</v>
+      </c>
+      <c r="D32" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="E32" t="s" s="0">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="s" s="0">
+        <v>347</v>
+      </c>
+      <c r="B33" t="s" s="0">
+        <v>348</v>
+      </c>
+      <c r="C33" t="s" s="0">
+        <v>349</v>
+      </c>
+      <c r="D33" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="E33" t="s" s="0">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="s" s="0">
+        <v>350</v>
+      </c>
+      <c r="B34" t="s" s="0">
+        <v>351</v>
+      </c>
+      <c r="C34" t="s" s="0">
+        <v>352</v>
+      </c>
+      <c r="D34" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="E34" t="s" s="0">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="s" s="0">
+        <v>353</v>
+      </c>
+      <c r="B35" t="s" s="0">
+        <v>354</v>
+      </c>
+      <c r="C35" t="s" s="0">
+        <v>355</v>
+      </c>
+      <c r="D35" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="E35" t="s" s="0">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="s" s="0">
+        <v>356</v>
+      </c>
+      <c r="B36" t="s" s="0">
+        <v>357</v>
+      </c>
+      <c r="C36" t="s" s="0">
+        <v>358</v>
+      </c>
+      <c r="D36" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="E36" t="s" s="0">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="s" s="0">
+        <v>359</v>
+      </c>
+      <c r="B37" t="s" s="0">
+        <v>360</v>
+      </c>
+      <c r="C37" t="s" s="0">
+        <v>361</v>
+      </c>
+      <c r="D37" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="E37" t="s" s="0">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="s" s="0">
+        <v>362</v>
+      </c>
+      <c r="B38" t="s" s="0">
+        <v>363</v>
+      </c>
+      <c r="C38" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="D38" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="E38" t="s" s="0">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="s" s="0">
+        <v>365</v>
+      </c>
+      <c r="B39" t="s" s="0">
+        <v>366</v>
+      </c>
+      <c r="C39" t="s" s="0">
+        <v>367</v>
+      </c>
+      <c r="D39" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="E39" t="s" s="0">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="s" s="0">
+        <v>368</v>
+      </c>
+      <c r="B40" t="s" s="0">
+        <v>369</v>
+      </c>
+      <c r="C40" t="s" s="0">
+        <v>370</v>
+      </c>
+      <c r="D40" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="E40" t="s" s="0">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="s" s="0">
+        <v>371</v>
+      </c>
+      <c r="B41" t="s" s="0">
+        <v>372</v>
+      </c>
+      <c r="C41" t="s" s="0">
+        <v>373</v>
+      </c>
+      <c r="D41" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="E41" t="s" s="0">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="s" s="0">
+        <v>374</v>
+      </c>
+      <c r="B42" t="s" s="0">
+        <v>375</v>
+      </c>
+      <c r="C42" t="s" s="0">
+        <v>376</v>
+      </c>
+      <c r="D42" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="E42" t="s" s="0">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="s" s="0">
+        <v>377</v>
+      </c>
+      <c r="B43" t="s" s="0">
+        <v>378</v>
+      </c>
+      <c r="C43" t="s" s="0">
+        <v>379</v>
+      </c>
+      <c r="D43" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="E43" t="s" s="0">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="s" s="0">
+        <v>380</v>
+      </c>
+      <c r="B44" t="s" s="0">
+        <v>381</v>
+      </c>
+      <c r="C44" t="s" s="0">
+        <v>382</v>
+      </c>
+      <c r="D44" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="E44" t="s" s="0">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="s" s="0">
+        <v>383</v>
+      </c>
+      <c r="B45" t="s" s="0">
+        <v>384</v>
+      </c>
+      <c r="C45" t="s" s="0">
+        <v>385</v>
+      </c>
+      <c r="D45" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="E45" t="s" s="0">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="s" s="0">
+        <v>386</v>
+      </c>
+      <c r="B46" t="s" s="0">
+        <v>387</v>
+      </c>
+      <c r="C46" t="s" s="0">
+        <v>388</v>
+      </c>
+      <c r="D46" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="E46" t="s" s="0">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="s" s="0">
+        <v>389</v>
+      </c>
+      <c r="B47" t="s" s="0">
+        <v>390</v>
+      </c>
+      <c r="C47" t="s" s="0">
+        <v>391</v>
+      </c>
+      <c r="D47" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="E47" t="s" s="0">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="s" s="0">
+        <v>392</v>
+      </c>
+      <c r="B48" t="s" s="0">
+        <v>393</v>
+      </c>
+      <c r="C48" t="s" s="0">
+        <v>394</v>
+      </c>
+      <c r="D48" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="E48" t="s" s="0">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="s" s="0">
+        <v>395</v>
+      </c>
+      <c r="B49" t="s" s="0">
+        <v>396</v>
+      </c>
+      <c r="C49" t="s" s="0">
+        <v>397</v>
+      </c>
+      <c r="D49" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="E49" t="s" s="0">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="s" s="0">
+        <v>398</v>
+      </c>
+      <c r="B50" t="s" s="0">
+        <v>399</v>
+      </c>
+      <c r="C50" t="s" s="0">
+        <v>400</v>
+      </c>
+      <c r="D50" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="E50" t="s" s="0">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="s" s="0">
+        <v>401</v>
+      </c>
+      <c r="B51" t="s" s="0">
+        <v>402</v>
+      </c>
+      <c r="C51" t="s" s="0">
+        <v>403</v>
+      </c>
+      <c r="D51" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="E51" t="s" s="0">
+        <v>65</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Bulk investment: AdviceStatus logging, Send OTP fix, locator updates, README update
</commit_message>
<xml_diff>
--- a/src/main/resources/testdata.xlsx
+++ b/src/main/resources/testdata.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11431" uniqueCount="539">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12961" uniqueCount="539">
   <si>
     <t>Key</t>
   </si>
@@ -1641,7 +1641,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="0"/>
-  <fonts count="25" x14ac:knownFonts="1">
+  <fonts count="31" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -1659,6 +1659,36 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -1791,7 +1821,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -1822,6 +1852,12 @@
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="true"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="true"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="true"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2412,31 +2448,31 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="s" s="25">
+      <c r="A1" t="s" s="31">
         <v>46</v>
       </c>
-      <c r="B1" t="s" s="25">
+      <c r="B1" t="s" s="31">
         <v>60</v>
       </c>
-      <c r="C1" t="s" s="25">
+      <c r="C1" t="s" s="31">
         <v>61</v>
       </c>
-      <c r="D1" t="s" s="25">
+      <c r="D1" t="s" s="31">
         <v>62</v>
       </c>
-      <c r="E1" t="s" s="25">
+      <c r="E1" t="s" s="31">
         <v>63</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>256</v>
+        <v>332</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>257</v>
+        <v>333</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>258</v>
+        <v>334</v>
       </c>
       <c r="D2" t="s" s="0">
         <v>64</v>
@@ -2447,13 +2483,13 @@
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>259</v>
+        <v>335</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>260</v>
+        <v>336</v>
       </c>
       <c r="C3" t="s" s="0">
-        <v>261</v>
+        <v>337</v>
       </c>
       <c r="D3" t="s" s="0">
         <v>64</v>
@@ -2464,13 +2500,13 @@
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>262</v>
+        <v>338</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>263</v>
+        <v>339</v>
       </c>
       <c r="C4" t="s" s="0">
-        <v>264</v>
+        <v>340</v>
       </c>
       <c r="D4" t="s" s="0">
         <v>64</v>
@@ -2481,13 +2517,13 @@
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>265</v>
+        <v>344</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>266</v>
+        <v>345</v>
       </c>
       <c r="C5" t="s" s="0">
-        <v>267</v>
+        <v>346</v>
       </c>
       <c r="D5" t="s" s="0">
         <v>64</v>
@@ -2498,13 +2534,13 @@
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>268</v>
+        <v>347</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>269</v>
+        <v>348</v>
       </c>
       <c r="C6" t="s" s="0">
-        <v>270</v>
+        <v>349</v>
       </c>
       <c r="D6" t="s" s="0">
         <v>64</v>
@@ -2515,13 +2551,13 @@
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>271</v>
+        <v>350</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>272</v>
+        <v>351</v>
       </c>
       <c r="C7" t="s" s="0">
-        <v>273</v>
+        <v>352</v>
       </c>
       <c r="D7" t="s" s="0">
         <v>64</v>
@@ -2532,13 +2568,13 @@
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>274</v>
+        <v>353</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>275</v>
+        <v>354</v>
       </c>
       <c r="C8" t="s" s="0">
-        <v>276</v>
+        <v>355</v>
       </c>
       <c r="D8" t="s" s="0">
         <v>64</v>
@@ -2549,13 +2585,13 @@
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
-        <v>277</v>
+        <v>356</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>278</v>
+        <v>357</v>
       </c>
       <c r="C9" t="s" s="0">
-        <v>279</v>
+        <v>358</v>
       </c>
       <c r="D9" t="s" s="0">
         <v>64</v>
@@ -2566,13 +2602,13 @@
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
-        <v>280</v>
+        <v>359</v>
       </c>
       <c r="B10" t="s" s="0">
-        <v>281</v>
+        <v>360</v>
       </c>
       <c r="C10" t="s" s="0">
-        <v>282</v>
+        <v>361</v>
       </c>
       <c r="D10" t="s" s="0">
         <v>64</v>
@@ -2583,13 +2619,13 @@
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
-        <v>283</v>
+        <v>362</v>
       </c>
       <c r="B11" t="s" s="0">
-        <v>284</v>
+        <v>363</v>
       </c>
       <c r="C11" t="s" s="0">
-        <v>285</v>
+        <v>364</v>
       </c>
       <c r="D11" t="s" s="0">
         <v>64</v>
@@ -2600,13 +2636,13 @@
     </row>
     <row r="12">
       <c r="A12" t="s" s="0">
-        <v>286</v>
+        <v>365</v>
       </c>
       <c r="B12" t="s" s="0">
-        <v>287</v>
+        <v>366</v>
       </c>
       <c r="C12" t="s" s="0">
-        <v>288</v>
+        <v>367</v>
       </c>
       <c r="D12" t="s" s="0">
         <v>64</v>
@@ -2617,13 +2653,13 @@
     </row>
     <row r="13">
       <c r="A13" t="s" s="0">
-        <v>289</v>
+        <v>368</v>
       </c>
       <c r="B13" t="s" s="0">
-        <v>290</v>
+        <v>369</v>
       </c>
       <c r="C13" t="s" s="0">
-        <v>291</v>
+        <v>370</v>
       </c>
       <c r="D13" t="s" s="0">
         <v>64</v>
@@ -2634,13 +2670,13 @@
     </row>
     <row r="14">
       <c r="A14" t="s" s="0">
-        <v>292</v>
+        <v>371</v>
       </c>
       <c r="B14" t="s" s="0">
-        <v>293</v>
+        <v>372</v>
       </c>
       <c r="C14" t="s" s="0">
-        <v>294</v>
+        <v>373</v>
       </c>
       <c r="D14" t="s" s="0">
         <v>64</v>
@@ -2651,13 +2687,13 @@
     </row>
     <row r="15">
       <c r="A15" t="s" s="0">
-        <v>295</v>
+        <v>374</v>
       </c>
       <c r="B15" t="s" s="0">
-        <v>296</v>
+        <v>375</v>
       </c>
       <c r="C15" t="s" s="0">
-        <v>297</v>
+        <v>376</v>
       </c>
       <c r="D15" t="s" s="0">
         <v>64</v>
@@ -2668,13 +2704,13 @@
     </row>
     <row r="16">
       <c r="A16" t="s" s="0">
-        <v>298</v>
+        <v>377</v>
       </c>
       <c r="B16" t="s" s="0">
-        <v>299</v>
+        <v>378</v>
       </c>
       <c r="C16" t="s" s="0">
-        <v>300</v>
+        <v>379</v>
       </c>
       <c r="D16" t="s" s="0">
         <v>64</v>
@@ -2685,13 +2721,13 @@
     </row>
     <row r="17">
       <c r="A17" t="s" s="0">
-        <v>301</v>
+        <v>380</v>
       </c>
       <c r="B17" t="s" s="0">
-        <v>302</v>
+        <v>381</v>
       </c>
       <c r="C17" t="s" s="0">
-        <v>303</v>
+        <v>382</v>
       </c>
       <c r="D17" t="s" s="0">
         <v>64</v>
@@ -2702,13 +2738,13 @@
     </row>
     <row r="18">
       <c r="A18" t="s" s="0">
-        <v>304</v>
+        <v>383</v>
       </c>
       <c r="B18" t="s" s="0">
-        <v>305</v>
+        <v>384</v>
       </c>
       <c r="C18" t="s" s="0">
-        <v>306</v>
+        <v>385</v>
       </c>
       <c r="D18" t="s" s="0">
         <v>64</v>
@@ -2719,13 +2755,13 @@
     </row>
     <row r="19">
       <c r="A19" t="s" s="0">
-        <v>307</v>
+        <v>386</v>
       </c>
       <c r="B19" t="s" s="0">
-        <v>302</v>
+        <v>387</v>
       </c>
       <c r="C19" t="s" s="0">
-        <v>303</v>
+        <v>388</v>
       </c>
       <c r="D19" t="s" s="0">
         <v>64</v>
@@ -2736,13 +2772,13 @@
     </row>
     <row r="20">
       <c r="A20" t="s" s="0">
-        <v>308</v>
+        <v>389</v>
       </c>
       <c r="B20" t="s" s="0">
-        <v>309</v>
+        <v>390</v>
       </c>
       <c r="C20" t="s" s="0">
-        <v>310</v>
+        <v>391</v>
       </c>
       <c r="D20" t="s" s="0">
         <v>64</v>
@@ -2753,13 +2789,13 @@
     </row>
     <row r="21">
       <c r="A21" t="s" s="0">
-        <v>311</v>
+        <v>392</v>
       </c>
       <c r="B21" t="s" s="0">
-        <v>312</v>
+        <v>393</v>
       </c>
       <c r="C21" t="s" s="0">
-        <v>313</v>
+        <v>394</v>
       </c>
       <c r="D21" t="s" s="0">
         <v>64</v>
@@ -2770,13 +2806,13 @@
     </row>
     <row r="22">
       <c r="A22" t="s" s="0">
-        <v>314</v>
+        <v>395</v>
       </c>
       <c r="B22" t="s" s="0">
-        <v>315</v>
+        <v>396</v>
       </c>
       <c r="C22" t="s" s="0">
-        <v>316</v>
+        <v>397</v>
       </c>
       <c r="D22" t="s" s="0">
         <v>64</v>
@@ -2787,13 +2823,13 @@
     </row>
     <row r="23">
       <c r="A23" t="s" s="0">
-        <v>317</v>
+        <v>398</v>
       </c>
       <c r="B23" t="s" s="0">
-        <v>318</v>
+        <v>399</v>
       </c>
       <c r="C23" t="s" s="0">
-        <v>319</v>
+        <v>400</v>
       </c>
       <c r="D23" t="s" s="0">
         <v>64</v>
@@ -2804,13 +2840,13 @@
     </row>
     <row r="24">
       <c r="A24" t="s" s="0">
-        <v>320</v>
+        <v>401</v>
       </c>
       <c r="B24" t="s" s="0">
-        <v>321</v>
+        <v>402</v>
       </c>
       <c r="C24" t="s" s="0">
-        <v>322</v>
+        <v>403</v>
       </c>
       <c r="D24" t="s" s="0">
         <v>64</v>
@@ -2821,13 +2857,13 @@
     </row>
     <row r="25">
       <c r="A25" t="s" s="0">
-        <v>323</v>
+        <v>404</v>
       </c>
       <c r="B25" t="s" s="0">
-        <v>324</v>
+        <v>405</v>
       </c>
       <c r="C25" t="s" s="0">
-        <v>325</v>
+        <v>406</v>
       </c>
       <c r="D25" t="s" s="0">
         <v>64</v>
@@ -2838,13 +2874,13 @@
     </row>
     <row r="26">
       <c r="A26" t="s" s="0">
-        <v>326</v>
+        <v>407</v>
       </c>
       <c r="B26" t="s" s="0">
-        <v>327</v>
+        <v>408</v>
       </c>
       <c r="C26" t="s" s="0">
-        <v>328</v>
+        <v>409</v>
       </c>
       <c r="D26" t="s" s="0">
         <v>64</v>
@@ -2855,13 +2891,13 @@
     </row>
     <row r="27">
       <c r="A27" t="s" s="0">
-        <v>329</v>
+        <v>410</v>
       </c>
       <c r="B27" t="s" s="0">
-        <v>330</v>
+        <v>411</v>
       </c>
       <c r="C27" t="s" s="0">
-        <v>331</v>
+        <v>412</v>
       </c>
       <c r="D27" t="s" s="0">
         <v>64</v>
@@ -2872,13 +2908,13 @@
     </row>
     <row r="28">
       <c r="A28" t="s" s="0">
-        <v>332</v>
+        <v>413</v>
       </c>
       <c r="B28" t="s" s="0">
-        <v>333</v>
+        <v>414</v>
       </c>
       <c r="C28" t="s" s="0">
-        <v>334</v>
+        <v>415</v>
       </c>
       <c r="D28" t="s" s="0">
         <v>64</v>
@@ -2889,13 +2925,13 @@
     </row>
     <row r="29">
       <c r="A29" t="s" s="0">
-        <v>335</v>
+        <v>416</v>
       </c>
       <c r="B29" t="s" s="0">
-        <v>336</v>
+        <v>417</v>
       </c>
       <c r="C29" t="s" s="0">
-        <v>337</v>
+        <v>418</v>
       </c>
       <c r="D29" t="s" s="0">
         <v>64</v>
@@ -2906,13 +2942,13 @@
     </row>
     <row r="30">
       <c r="A30" t="s" s="0">
-        <v>338</v>
+        <v>419</v>
       </c>
       <c r="B30" t="s" s="0">
-        <v>339</v>
+        <v>420</v>
       </c>
       <c r="C30" t="s" s="0">
-        <v>340</v>
+        <v>421</v>
       </c>
       <c r="D30" t="s" s="0">
         <v>64</v>
@@ -2923,13 +2959,13 @@
     </row>
     <row r="31">
       <c r="A31" t="s" s="0">
-        <v>341</v>
+        <v>422</v>
       </c>
       <c r="B31" t="s" s="0">
-        <v>342</v>
+        <v>423</v>
       </c>
       <c r="C31" t="s" s="0">
-        <v>343</v>
+        <v>424</v>
       </c>
       <c r="D31" t="s" s="0">
         <v>64</v>
@@ -2940,13 +2976,13 @@
     </row>
     <row r="32">
       <c r="A32" t="s" s="0">
-        <v>344</v>
+        <v>425</v>
       </c>
       <c r="B32" t="s" s="0">
-        <v>345</v>
+        <v>426</v>
       </c>
       <c r="C32" t="s" s="0">
-        <v>346</v>
+        <v>427</v>
       </c>
       <c r="D32" t="s" s="0">
         <v>64</v>
@@ -2957,13 +2993,13 @@
     </row>
     <row r="33">
       <c r="A33" t="s" s="0">
-        <v>347</v>
+        <v>431</v>
       </c>
       <c r="B33" t="s" s="0">
-        <v>348</v>
+        <v>432</v>
       </c>
       <c r="C33" t="s" s="0">
-        <v>349</v>
+        <v>433</v>
       </c>
       <c r="D33" t="s" s="0">
         <v>64</v>
@@ -2974,13 +3010,13 @@
     </row>
     <row r="34">
       <c r="A34" t="s" s="0">
-        <v>350</v>
+        <v>434</v>
       </c>
       <c r="B34" t="s" s="0">
-        <v>351</v>
+        <v>435</v>
       </c>
       <c r="C34" t="s" s="0">
-        <v>352</v>
+        <v>436</v>
       </c>
       <c r="D34" t="s" s="0">
         <v>64</v>
@@ -2991,13 +3027,13 @@
     </row>
     <row r="35">
       <c r="A35" t="s" s="0">
-        <v>353</v>
+        <v>437</v>
       </c>
       <c r="B35" t="s" s="0">
-        <v>354</v>
+        <v>438</v>
       </c>
       <c r="C35" t="s" s="0">
-        <v>355</v>
+        <v>439</v>
       </c>
       <c r="D35" t="s" s="0">
         <v>64</v>
@@ -3008,13 +3044,13 @@
     </row>
     <row r="36">
       <c r="A36" t="s" s="0">
-        <v>356</v>
+        <v>440</v>
       </c>
       <c r="B36" t="s" s="0">
-        <v>357</v>
+        <v>441</v>
       </c>
       <c r="C36" t="s" s="0">
-        <v>358</v>
+        <v>442</v>
       </c>
       <c r="D36" t="s" s="0">
         <v>64</v>
@@ -3025,13 +3061,13 @@
     </row>
     <row r="37">
       <c r="A37" t="s" s="0">
-        <v>359</v>
+        <v>443</v>
       </c>
       <c r="B37" t="s" s="0">
-        <v>360</v>
+        <v>444</v>
       </c>
       <c r="C37" t="s" s="0">
-        <v>361</v>
+        <v>445</v>
       </c>
       <c r="D37" t="s" s="0">
         <v>64</v>
@@ -3042,13 +3078,13 @@
     </row>
     <row r="38">
       <c r="A38" t="s" s="0">
-        <v>362</v>
+        <v>446</v>
       </c>
       <c r="B38" t="s" s="0">
-        <v>363</v>
+        <v>447</v>
       </c>
       <c r="C38" t="s" s="0">
-        <v>364</v>
+        <v>448</v>
       </c>
       <c r="D38" t="s" s="0">
         <v>64</v>
@@ -3059,13 +3095,13 @@
     </row>
     <row r="39">
       <c r="A39" t="s" s="0">
-        <v>365</v>
+        <v>449</v>
       </c>
       <c r="B39" t="s" s="0">
-        <v>366</v>
+        <v>450</v>
       </c>
       <c r="C39" t="s" s="0">
-        <v>367</v>
+        <v>451</v>
       </c>
       <c r="D39" t="s" s="0">
         <v>64</v>
@@ -3076,13 +3112,13 @@
     </row>
     <row r="40">
       <c r="A40" t="s" s="0">
-        <v>368</v>
+        <v>452</v>
       </c>
       <c r="B40" t="s" s="0">
-        <v>369</v>
+        <v>453</v>
       </c>
       <c r="C40" t="s" s="0">
-        <v>370</v>
+        <v>454</v>
       </c>
       <c r="D40" t="s" s="0">
         <v>64</v>
@@ -3093,13 +3129,13 @@
     </row>
     <row r="41">
       <c r="A41" t="s" s="0">
-        <v>371</v>
+        <v>455</v>
       </c>
       <c r="B41" t="s" s="0">
-        <v>372</v>
+        <v>456</v>
       </c>
       <c r="C41" t="s" s="0">
-        <v>373</v>
+        <v>457</v>
       </c>
       <c r="D41" t="s" s="0">
         <v>64</v>
@@ -3110,13 +3146,13 @@
     </row>
     <row r="42">
       <c r="A42" t="s" s="0">
-        <v>374</v>
+        <v>458</v>
       </c>
       <c r="B42" t="s" s="0">
-        <v>375</v>
+        <v>459</v>
       </c>
       <c r="C42" t="s" s="0">
-        <v>376</v>
+        <v>460</v>
       </c>
       <c r="D42" t="s" s="0">
         <v>64</v>
@@ -3127,13 +3163,13 @@
     </row>
     <row r="43">
       <c r="A43" t="s" s="0">
-        <v>377</v>
+        <v>461</v>
       </c>
       <c r="B43" t="s" s="0">
-        <v>378</v>
+        <v>462</v>
       </c>
       <c r="C43" t="s" s="0">
-        <v>379</v>
+        <v>463</v>
       </c>
       <c r="D43" t="s" s="0">
         <v>64</v>
@@ -3144,13 +3180,13 @@
     </row>
     <row r="44">
       <c r="A44" t="s" s="0">
-        <v>380</v>
+        <v>464</v>
       </c>
       <c r="B44" t="s" s="0">
-        <v>381</v>
+        <v>465</v>
       </c>
       <c r="C44" t="s" s="0">
-        <v>382</v>
+        <v>466</v>
       </c>
       <c r="D44" t="s" s="0">
         <v>64</v>
@@ -3161,13 +3197,13 @@
     </row>
     <row r="45">
       <c r="A45" t="s" s="0">
-        <v>383</v>
+        <v>470</v>
       </c>
       <c r="B45" t="s" s="0">
-        <v>384</v>
+        <v>471</v>
       </c>
       <c r="C45" t="s" s="0">
-        <v>385</v>
+        <v>472</v>
       </c>
       <c r="D45" t="s" s="0">
         <v>64</v>
@@ -3178,13 +3214,13 @@
     </row>
     <row r="46">
       <c r="A46" t="s" s="0">
-        <v>386</v>
+        <v>473</v>
       </c>
       <c r="B46" t="s" s="0">
-        <v>387</v>
+        <v>474</v>
       </c>
       <c r="C46" t="s" s="0">
-        <v>388</v>
+        <v>475</v>
       </c>
       <c r="D46" t="s" s="0">
         <v>64</v>
@@ -3195,13 +3231,13 @@
     </row>
     <row r="47">
       <c r="A47" t="s" s="0">
-        <v>389</v>
+        <v>476</v>
       </c>
       <c r="B47" t="s" s="0">
-        <v>390</v>
+        <v>477</v>
       </c>
       <c r="C47" t="s" s="0">
-        <v>391</v>
+        <v>478</v>
       </c>
       <c r="D47" t="s" s="0">
         <v>64</v>
@@ -3212,13 +3248,13 @@
     </row>
     <row r="48">
       <c r="A48" t="s" s="0">
-        <v>392</v>
+        <v>479</v>
       </c>
       <c r="B48" t="s" s="0">
-        <v>393</v>
+        <v>480</v>
       </c>
       <c r="C48" t="s" s="0">
-        <v>394</v>
+        <v>481</v>
       </c>
       <c r="D48" t="s" s="0">
         <v>64</v>
@@ -3229,13 +3265,13 @@
     </row>
     <row r="49">
       <c r="A49" t="s" s="0">
-        <v>395</v>
+        <v>482</v>
       </c>
       <c r="B49" t="s" s="0">
-        <v>396</v>
+        <v>483</v>
       </c>
       <c r="C49" t="s" s="0">
-        <v>397</v>
+        <v>484</v>
       </c>
       <c r="D49" t="s" s="0">
         <v>64</v>
@@ -3246,13 +3282,13 @@
     </row>
     <row r="50">
       <c r="A50" t="s" s="0">
-        <v>398</v>
+        <v>485</v>
       </c>
       <c r="B50" t="s" s="0">
-        <v>399</v>
+        <v>486</v>
       </c>
       <c r="C50" t="s" s="0">
-        <v>400</v>
+        <v>487</v>
       </c>
       <c r="D50" t="s" s="0">
         <v>64</v>
@@ -3263,13 +3299,13 @@
     </row>
     <row r="51">
       <c r="A51" t="s" s="0">
-        <v>401</v>
+        <v>488</v>
       </c>
       <c r="B51" t="s" s="0">
-        <v>402</v>
+        <v>489</v>
       </c>
       <c r="C51" t="s" s="0">
-        <v>403</v>
+        <v>490</v>
       </c>
       <c r="D51" t="s" s="0">
         <v>64</v>

</xml_diff>

<commit_message>
Bulk investment: remove debug logs, clean Send OTP click, fix popup dismiss timeout
</commit_message>
<xml_diff>
--- a/src/main/resources/testdata.xlsx
+++ b/src/main/resources/testdata.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12961" uniqueCount="539">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13216" uniqueCount="539">
   <si>
     <t>Key</t>
   </si>
@@ -1641,7 +1641,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="0"/>
-  <fonts count="31" x14ac:knownFonts="1">
+  <fonts count="32" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -1659,6 +1659,11 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -1821,7 +1826,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -1858,6 +1863,7 @@
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="true"/>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="true"/>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="true"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2448,31 +2454,31 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="s" s="31">
+      <c r="A1" t="s" s="32">
         <v>46</v>
       </c>
-      <c r="B1" t="s" s="31">
+      <c r="B1" t="s" s="32">
         <v>60</v>
       </c>
-      <c r="C1" t="s" s="31">
+      <c r="C1" t="s" s="32">
         <v>61</v>
       </c>
-      <c r="D1" t="s" s="31">
+      <c r="D1" t="s" s="32">
         <v>62</v>
       </c>
-      <c r="E1" t="s" s="31">
+      <c r="E1" t="s" s="32">
         <v>63</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>332</v>
+        <v>347</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>333</v>
+        <v>348</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>334</v>
+        <v>349</v>
       </c>
       <c r="D2" t="s" s="0">
         <v>64</v>
@@ -2483,13 +2489,13 @@
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>335</v>
+        <v>350</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>336</v>
+        <v>351</v>
       </c>
       <c r="C3" t="s" s="0">
-        <v>337</v>
+        <v>352</v>
       </c>
       <c r="D3" t="s" s="0">
         <v>64</v>
@@ -2500,13 +2506,13 @@
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>338</v>
+        <v>353</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>339</v>
+        <v>354</v>
       </c>
       <c r="C4" t="s" s="0">
-        <v>340</v>
+        <v>355</v>
       </c>
       <c r="D4" t="s" s="0">
         <v>64</v>
@@ -2517,13 +2523,13 @@
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>344</v>
+        <v>356</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>345</v>
+        <v>357</v>
       </c>
       <c r="C5" t="s" s="0">
-        <v>346</v>
+        <v>358</v>
       </c>
       <c r="D5" t="s" s="0">
         <v>64</v>
@@ -2534,13 +2540,13 @@
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>347</v>
+        <v>359</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>348</v>
+        <v>360</v>
       </c>
       <c r="C6" t="s" s="0">
-        <v>349</v>
+        <v>361</v>
       </c>
       <c r="D6" t="s" s="0">
         <v>64</v>
@@ -2551,13 +2557,13 @@
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>350</v>
+        <v>362</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>351</v>
+        <v>363</v>
       </c>
       <c r="C7" t="s" s="0">
-        <v>352</v>
+        <v>364</v>
       </c>
       <c r="D7" t="s" s="0">
         <v>64</v>
@@ -2568,13 +2574,13 @@
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>353</v>
+        <v>365</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>354</v>
+        <v>366</v>
       </c>
       <c r="C8" t="s" s="0">
-        <v>355</v>
+        <v>367</v>
       </c>
       <c r="D8" t="s" s="0">
         <v>64</v>
@@ -2585,13 +2591,13 @@
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
-        <v>356</v>
+        <v>368</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>357</v>
+        <v>369</v>
       </c>
       <c r="C9" t="s" s="0">
-        <v>358</v>
+        <v>370</v>
       </c>
       <c r="D9" t="s" s="0">
         <v>64</v>
@@ -2602,13 +2608,13 @@
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
-        <v>359</v>
+        <v>371</v>
       </c>
       <c r="B10" t="s" s="0">
-        <v>360</v>
+        <v>372</v>
       </c>
       <c r="C10" t="s" s="0">
-        <v>361</v>
+        <v>373</v>
       </c>
       <c r="D10" t="s" s="0">
         <v>64</v>
@@ -2619,13 +2625,13 @@
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
-        <v>362</v>
+        <v>374</v>
       </c>
       <c r="B11" t="s" s="0">
-        <v>363</v>
+        <v>375</v>
       </c>
       <c r="C11" t="s" s="0">
-        <v>364</v>
+        <v>376</v>
       </c>
       <c r="D11" t="s" s="0">
         <v>64</v>
@@ -2636,13 +2642,13 @@
     </row>
     <row r="12">
       <c r="A12" t="s" s="0">
-        <v>365</v>
+        <v>377</v>
       </c>
       <c r="B12" t="s" s="0">
-        <v>366</v>
+        <v>378</v>
       </c>
       <c r="C12" t="s" s="0">
-        <v>367</v>
+        <v>379</v>
       </c>
       <c r="D12" t="s" s="0">
         <v>64</v>
@@ -2653,13 +2659,13 @@
     </row>
     <row r="13">
       <c r="A13" t="s" s="0">
-        <v>368</v>
+        <v>380</v>
       </c>
       <c r="B13" t="s" s="0">
-        <v>369</v>
+        <v>381</v>
       </c>
       <c r="C13" t="s" s="0">
-        <v>370</v>
+        <v>382</v>
       </c>
       <c r="D13" t="s" s="0">
         <v>64</v>
@@ -2670,13 +2676,13 @@
     </row>
     <row r="14">
       <c r="A14" t="s" s="0">
-        <v>371</v>
+        <v>383</v>
       </c>
       <c r="B14" t="s" s="0">
-        <v>372</v>
+        <v>384</v>
       </c>
       <c r="C14" t="s" s="0">
-        <v>373</v>
+        <v>385</v>
       </c>
       <c r="D14" t="s" s="0">
         <v>64</v>
@@ -2687,13 +2693,13 @@
     </row>
     <row r="15">
       <c r="A15" t="s" s="0">
-        <v>374</v>
+        <v>386</v>
       </c>
       <c r="B15" t="s" s="0">
-        <v>375</v>
+        <v>387</v>
       </c>
       <c r="C15" t="s" s="0">
-        <v>376</v>
+        <v>388</v>
       </c>
       <c r="D15" t="s" s="0">
         <v>64</v>
@@ -2704,13 +2710,13 @@
     </row>
     <row r="16">
       <c r="A16" t="s" s="0">
-        <v>377</v>
+        <v>389</v>
       </c>
       <c r="B16" t="s" s="0">
-        <v>378</v>
+        <v>390</v>
       </c>
       <c r="C16" t="s" s="0">
-        <v>379</v>
+        <v>391</v>
       </c>
       <c r="D16" t="s" s="0">
         <v>64</v>
@@ -2721,13 +2727,13 @@
     </row>
     <row r="17">
       <c r="A17" t="s" s="0">
-        <v>380</v>
+        <v>392</v>
       </c>
       <c r="B17" t="s" s="0">
-        <v>381</v>
+        <v>393</v>
       </c>
       <c r="C17" t="s" s="0">
-        <v>382</v>
+        <v>394</v>
       </c>
       <c r="D17" t="s" s="0">
         <v>64</v>
@@ -2738,13 +2744,13 @@
     </row>
     <row r="18">
       <c r="A18" t="s" s="0">
-        <v>383</v>
+        <v>395</v>
       </c>
       <c r="B18" t="s" s="0">
-        <v>384</v>
+        <v>396</v>
       </c>
       <c r="C18" t="s" s="0">
-        <v>385</v>
+        <v>397</v>
       </c>
       <c r="D18" t="s" s="0">
         <v>64</v>
@@ -2755,13 +2761,13 @@
     </row>
     <row r="19">
       <c r="A19" t="s" s="0">
-        <v>386</v>
+        <v>398</v>
       </c>
       <c r="B19" t="s" s="0">
-        <v>387</v>
+        <v>399</v>
       </c>
       <c r="C19" t="s" s="0">
-        <v>388</v>
+        <v>400</v>
       </c>
       <c r="D19" t="s" s="0">
         <v>64</v>
@@ -2772,13 +2778,13 @@
     </row>
     <row r="20">
       <c r="A20" t="s" s="0">
-        <v>389</v>
+        <v>401</v>
       </c>
       <c r="B20" t="s" s="0">
-        <v>390</v>
+        <v>402</v>
       </c>
       <c r="C20" t="s" s="0">
-        <v>391</v>
+        <v>403</v>
       </c>
       <c r="D20" t="s" s="0">
         <v>64</v>
@@ -2789,13 +2795,13 @@
     </row>
     <row r="21">
       <c r="A21" t="s" s="0">
-        <v>392</v>
+        <v>404</v>
       </c>
       <c r="B21" t="s" s="0">
-        <v>393</v>
+        <v>405</v>
       </c>
       <c r="C21" t="s" s="0">
-        <v>394</v>
+        <v>406</v>
       </c>
       <c r="D21" t="s" s="0">
         <v>64</v>
@@ -2806,13 +2812,13 @@
     </row>
     <row r="22">
       <c r="A22" t="s" s="0">
-        <v>395</v>
+        <v>407</v>
       </c>
       <c r="B22" t="s" s="0">
-        <v>396</v>
+        <v>408</v>
       </c>
       <c r="C22" t="s" s="0">
-        <v>397</v>
+        <v>409</v>
       </c>
       <c r="D22" t="s" s="0">
         <v>64</v>
@@ -2823,13 +2829,13 @@
     </row>
     <row r="23">
       <c r="A23" t="s" s="0">
-        <v>398</v>
+        <v>410</v>
       </c>
       <c r="B23" t="s" s="0">
-        <v>399</v>
+        <v>411</v>
       </c>
       <c r="C23" t="s" s="0">
-        <v>400</v>
+        <v>412</v>
       </c>
       <c r="D23" t="s" s="0">
         <v>64</v>
@@ -2840,13 +2846,13 @@
     </row>
     <row r="24">
       <c r="A24" t="s" s="0">
-        <v>401</v>
+        <v>413</v>
       </c>
       <c r="B24" t="s" s="0">
-        <v>402</v>
+        <v>414</v>
       </c>
       <c r="C24" t="s" s="0">
-        <v>403</v>
+        <v>415</v>
       </c>
       <c r="D24" t="s" s="0">
         <v>64</v>
@@ -2857,13 +2863,13 @@
     </row>
     <row r="25">
       <c r="A25" t="s" s="0">
-        <v>404</v>
+        <v>416</v>
       </c>
       <c r="B25" t="s" s="0">
-        <v>405</v>
+        <v>417</v>
       </c>
       <c r="C25" t="s" s="0">
-        <v>406</v>
+        <v>418</v>
       </c>
       <c r="D25" t="s" s="0">
         <v>64</v>
@@ -2874,13 +2880,13 @@
     </row>
     <row r="26">
       <c r="A26" t="s" s="0">
-        <v>407</v>
+        <v>419</v>
       </c>
       <c r="B26" t="s" s="0">
-        <v>408</v>
+        <v>420</v>
       </c>
       <c r="C26" t="s" s="0">
-        <v>409</v>
+        <v>421</v>
       </c>
       <c r="D26" t="s" s="0">
         <v>64</v>
@@ -2891,13 +2897,13 @@
     </row>
     <row r="27">
       <c r="A27" t="s" s="0">
-        <v>410</v>
+        <v>422</v>
       </c>
       <c r="B27" t="s" s="0">
-        <v>411</v>
+        <v>423</v>
       </c>
       <c r="C27" t="s" s="0">
-        <v>412</v>
+        <v>424</v>
       </c>
       <c r="D27" t="s" s="0">
         <v>64</v>
@@ -2908,13 +2914,13 @@
     </row>
     <row r="28">
       <c r="A28" t="s" s="0">
-        <v>413</v>
+        <v>425</v>
       </c>
       <c r="B28" t="s" s="0">
-        <v>414</v>
+        <v>426</v>
       </c>
       <c r="C28" t="s" s="0">
-        <v>415</v>
+        <v>427</v>
       </c>
       <c r="D28" t="s" s="0">
         <v>64</v>
@@ -2925,13 +2931,13 @@
     </row>
     <row r="29">
       <c r="A29" t="s" s="0">
-        <v>416</v>
+        <v>431</v>
       </c>
       <c r="B29" t="s" s="0">
-        <v>417</v>
+        <v>432</v>
       </c>
       <c r="C29" t="s" s="0">
-        <v>418</v>
+        <v>433</v>
       </c>
       <c r="D29" t="s" s="0">
         <v>64</v>
@@ -2942,13 +2948,13 @@
     </row>
     <row r="30">
       <c r="A30" t="s" s="0">
-        <v>419</v>
+        <v>434</v>
       </c>
       <c r="B30" t="s" s="0">
-        <v>420</v>
+        <v>435</v>
       </c>
       <c r="C30" t="s" s="0">
-        <v>421</v>
+        <v>436</v>
       </c>
       <c r="D30" t="s" s="0">
         <v>64</v>
@@ -2959,13 +2965,13 @@
     </row>
     <row r="31">
       <c r="A31" t="s" s="0">
-        <v>422</v>
+        <v>437</v>
       </c>
       <c r="B31" t="s" s="0">
-        <v>423</v>
+        <v>438</v>
       </c>
       <c r="C31" t="s" s="0">
-        <v>424</v>
+        <v>439</v>
       </c>
       <c r="D31" t="s" s="0">
         <v>64</v>
@@ -2976,13 +2982,13 @@
     </row>
     <row r="32">
       <c r="A32" t="s" s="0">
-        <v>425</v>
+        <v>440</v>
       </c>
       <c r="B32" t="s" s="0">
-        <v>426</v>
+        <v>441</v>
       </c>
       <c r="C32" t="s" s="0">
-        <v>427</v>
+        <v>442</v>
       </c>
       <c r="D32" t="s" s="0">
         <v>64</v>
@@ -2993,13 +2999,13 @@
     </row>
     <row r="33">
       <c r="A33" t="s" s="0">
-        <v>431</v>
+        <v>443</v>
       </c>
       <c r="B33" t="s" s="0">
-        <v>432</v>
+        <v>444</v>
       </c>
       <c r="C33" t="s" s="0">
-        <v>433</v>
+        <v>445</v>
       </c>
       <c r="D33" t="s" s="0">
         <v>64</v>
@@ -3010,13 +3016,13 @@
     </row>
     <row r="34">
       <c r="A34" t="s" s="0">
-        <v>434</v>
+        <v>446</v>
       </c>
       <c r="B34" t="s" s="0">
-        <v>435</v>
+        <v>447</v>
       </c>
       <c r="C34" t="s" s="0">
-        <v>436</v>
+        <v>448</v>
       </c>
       <c r="D34" t="s" s="0">
         <v>64</v>
@@ -3027,13 +3033,13 @@
     </row>
     <row r="35">
       <c r="A35" t="s" s="0">
-        <v>437</v>
+        <v>449</v>
       </c>
       <c r="B35" t="s" s="0">
-        <v>438</v>
+        <v>450</v>
       </c>
       <c r="C35" t="s" s="0">
-        <v>439</v>
+        <v>451</v>
       </c>
       <c r="D35" t="s" s="0">
         <v>64</v>
@@ -3044,13 +3050,13 @@
     </row>
     <row r="36">
       <c r="A36" t="s" s="0">
-        <v>440</v>
+        <v>452</v>
       </c>
       <c r="B36" t="s" s="0">
-        <v>441</v>
+        <v>453</v>
       </c>
       <c r="C36" t="s" s="0">
-        <v>442</v>
+        <v>454</v>
       </c>
       <c r="D36" t="s" s="0">
         <v>64</v>
@@ -3061,13 +3067,13 @@
     </row>
     <row r="37">
       <c r="A37" t="s" s="0">
-        <v>443</v>
+        <v>455</v>
       </c>
       <c r="B37" t="s" s="0">
-        <v>444</v>
+        <v>456</v>
       </c>
       <c r="C37" t="s" s="0">
-        <v>445</v>
+        <v>457</v>
       </c>
       <c r="D37" t="s" s="0">
         <v>64</v>
@@ -3078,13 +3084,13 @@
     </row>
     <row r="38">
       <c r="A38" t="s" s="0">
-        <v>446</v>
+        <v>458</v>
       </c>
       <c r="B38" t="s" s="0">
-        <v>447</v>
+        <v>459</v>
       </c>
       <c r="C38" t="s" s="0">
-        <v>448</v>
+        <v>460</v>
       </c>
       <c r="D38" t="s" s="0">
         <v>64</v>
@@ -3095,13 +3101,13 @@
     </row>
     <row r="39">
       <c r="A39" t="s" s="0">
-        <v>449</v>
+        <v>461</v>
       </c>
       <c r="B39" t="s" s="0">
-        <v>450</v>
+        <v>462</v>
       </c>
       <c r="C39" t="s" s="0">
-        <v>451</v>
+        <v>463</v>
       </c>
       <c r="D39" t="s" s="0">
         <v>64</v>
@@ -3112,13 +3118,13 @@
     </row>
     <row r="40">
       <c r="A40" t="s" s="0">
-        <v>452</v>
+        <v>464</v>
       </c>
       <c r="B40" t="s" s="0">
-        <v>453</v>
+        <v>465</v>
       </c>
       <c r="C40" t="s" s="0">
-        <v>454</v>
+        <v>466</v>
       </c>
       <c r="D40" t="s" s="0">
         <v>64</v>
@@ -3129,13 +3135,13 @@
     </row>
     <row r="41">
       <c r="A41" t="s" s="0">
-        <v>455</v>
+        <v>470</v>
       </c>
       <c r="B41" t="s" s="0">
-        <v>456</v>
+        <v>471</v>
       </c>
       <c r="C41" t="s" s="0">
-        <v>457</v>
+        <v>472</v>
       </c>
       <c r="D41" t="s" s="0">
         <v>64</v>
@@ -3146,13 +3152,13 @@
     </row>
     <row r="42">
       <c r="A42" t="s" s="0">
-        <v>458</v>
+        <v>473</v>
       </c>
       <c r="B42" t="s" s="0">
-        <v>459</v>
+        <v>474</v>
       </c>
       <c r="C42" t="s" s="0">
-        <v>460</v>
+        <v>475</v>
       </c>
       <c r="D42" t="s" s="0">
         <v>64</v>
@@ -3163,13 +3169,13 @@
     </row>
     <row r="43">
       <c r="A43" t="s" s="0">
-        <v>461</v>
+        <v>476</v>
       </c>
       <c r="B43" t="s" s="0">
-        <v>462</v>
+        <v>477</v>
       </c>
       <c r="C43" t="s" s="0">
-        <v>463</v>
+        <v>478</v>
       </c>
       <c r="D43" t="s" s="0">
         <v>64</v>
@@ -3180,13 +3186,13 @@
     </row>
     <row r="44">
       <c r="A44" t="s" s="0">
-        <v>464</v>
+        <v>479</v>
       </c>
       <c r="B44" t="s" s="0">
-        <v>465</v>
+        <v>480</v>
       </c>
       <c r="C44" t="s" s="0">
-        <v>466</v>
+        <v>481</v>
       </c>
       <c r="D44" t="s" s="0">
         <v>64</v>
@@ -3197,13 +3203,13 @@
     </row>
     <row r="45">
       <c r="A45" t="s" s="0">
-        <v>470</v>
+        <v>482</v>
       </c>
       <c r="B45" t="s" s="0">
-        <v>471</v>
+        <v>483</v>
       </c>
       <c r="C45" t="s" s="0">
-        <v>472</v>
+        <v>484</v>
       </c>
       <c r="D45" t="s" s="0">
         <v>64</v>
@@ -3214,13 +3220,13 @@
     </row>
     <row r="46">
       <c r="A46" t="s" s="0">
-        <v>473</v>
+        <v>485</v>
       </c>
       <c r="B46" t="s" s="0">
-        <v>474</v>
+        <v>486</v>
       </c>
       <c r="C46" t="s" s="0">
-        <v>475</v>
+        <v>487</v>
       </c>
       <c r="D46" t="s" s="0">
         <v>64</v>
@@ -3231,13 +3237,13 @@
     </row>
     <row r="47">
       <c r="A47" t="s" s="0">
-        <v>476</v>
+        <v>488</v>
       </c>
       <c r="B47" t="s" s="0">
-        <v>477</v>
+        <v>489</v>
       </c>
       <c r="C47" t="s" s="0">
-        <v>478</v>
+        <v>490</v>
       </c>
       <c r="D47" t="s" s="0">
         <v>64</v>
@@ -3248,13 +3254,13 @@
     </row>
     <row r="48">
       <c r="A48" t="s" s="0">
-        <v>479</v>
+        <v>491</v>
       </c>
       <c r="B48" t="s" s="0">
-        <v>480</v>
+        <v>492</v>
       </c>
       <c r="C48" t="s" s="0">
-        <v>481</v>
+        <v>493</v>
       </c>
       <c r="D48" t="s" s="0">
         <v>64</v>
@@ -3265,13 +3271,13 @@
     </row>
     <row r="49">
       <c r="A49" t="s" s="0">
-        <v>482</v>
+        <v>494</v>
       </c>
       <c r="B49" t="s" s="0">
-        <v>483</v>
+        <v>495</v>
       </c>
       <c r="C49" t="s" s="0">
-        <v>484</v>
+        <v>496</v>
       </c>
       <c r="D49" t="s" s="0">
         <v>64</v>
@@ -3282,13 +3288,13 @@
     </row>
     <row r="50">
       <c r="A50" t="s" s="0">
-        <v>485</v>
+        <v>497</v>
       </c>
       <c r="B50" t="s" s="0">
-        <v>486</v>
+        <v>498</v>
       </c>
       <c r="C50" t="s" s="0">
-        <v>487</v>
+        <v>499</v>
       </c>
       <c r="D50" t="s" s="0">
         <v>64</v>
@@ -3299,13 +3305,13 @@
     </row>
     <row r="51">
       <c r="A51" t="s" s="0">
-        <v>488</v>
+        <v>500</v>
       </c>
       <c r="B51" t="s" s="0">
-        <v>489</v>
+        <v>501</v>
       </c>
       <c r="C51" t="s" s="0">
-        <v>490</v>
+        <v>502</v>
       </c>
       <c r="D51" t="s" s="0">
         <v>64</v>

</xml_diff>

<commit_message>
Add driver warmup, PROJECT_GUIDE.md fixes, BaseTest and DriverFactory updates
</commit_message>
<xml_diff>
--- a/src/main/resources/testdata.xlsx
+++ b/src/main/resources/testdata.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13216" uniqueCount="539">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14281" uniqueCount="581">
   <si>
     <t>Key</t>
   </si>
@@ -1634,6 +1634,132 @@
   </si>
   <si>
     <t>01/01/1964</t>
+  </si>
+  <si>
+    <t>BANB1247</t>
+  </si>
+  <si>
+    <t>1995-12-13</t>
+  </si>
+  <si>
+    <t>13/12/1995</t>
+  </si>
+  <si>
+    <t>BLLS1515</t>
+  </si>
+  <si>
+    <t>1993-10-09</t>
+  </si>
+  <si>
+    <t>09/10/1993</t>
+  </si>
+  <si>
+    <t>BRD1193</t>
+  </si>
+  <si>
+    <t>1957-11-18</t>
+  </si>
+  <si>
+    <t>18/11/1957</t>
+  </si>
+  <si>
+    <t>BRD1196</t>
+  </si>
+  <si>
+    <t>1974-02-09</t>
+  </si>
+  <si>
+    <t>09/02/1974</t>
+  </si>
+  <si>
+    <t>BRD462</t>
+  </si>
+  <si>
+    <t>1985-07-01</t>
+  </si>
+  <si>
+    <t>01/07/1985</t>
+  </si>
+  <si>
+    <t>BRD837</t>
+  </si>
+  <si>
+    <t>1998-06-17</t>
+  </si>
+  <si>
+    <t>17/06/1998</t>
+  </si>
+  <si>
+    <t>RETK2911</t>
+  </si>
+  <si>
+    <t>1998-07-22</t>
+  </si>
+  <si>
+    <t>22/07/1998</t>
+  </si>
+  <si>
+    <t>RETK2912</t>
+  </si>
+  <si>
+    <t>1985-03-04</t>
+  </si>
+  <si>
+    <t>04/03/1985</t>
+  </si>
+  <si>
+    <t>RETK2926</t>
+  </si>
+  <si>
+    <t>1980-01-01</t>
+  </si>
+  <si>
+    <t>01/01/1980</t>
+  </si>
+  <si>
+    <t>RETK2947</t>
+  </si>
+  <si>
+    <t>1983-06-22</t>
+  </si>
+  <si>
+    <t>22/06/1983</t>
+  </si>
+  <si>
+    <t>RETK2969</t>
+  </si>
+  <si>
+    <t>1992-06-06</t>
+  </si>
+  <si>
+    <t>06/06/1992</t>
+  </si>
+  <si>
+    <t>RETK2975</t>
+  </si>
+  <si>
+    <t>1980-12-30</t>
+  </si>
+  <si>
+    <t>30/12/1980</t>
+  </si>
+  <si>
+    <t>RETK2978</t>
+  </si>
+  <si>
+    <t>1990-03-15</t>
+  </si>
+  <si>
+    <t>15/03/1990</t>
+  </si>
+  <si>
+    <t>RETK2995</t>
+  </si>
+  <si>
+    <t>1992-05-13</t>
+  </si>
+  <si>
+    <t>13/05/1992</t>
   </si>
 </sst>
 </file>
@@ -1641,7 +1767,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="0"/>
-  <fonts count="32" x14ac:knownFonts="1">
+  <fonts count="35" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -1659,6 +1785,21 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -1826,7 +1967,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -1864,6 +2005,9 @@
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="true"/>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="true"/>
     <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="true"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2443,7 +2587,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E51"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="9.85546875" customWidth="true" bestFit="true"/>
@@ -2454,31 +2598,31 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="s" s="32">
+      <c r="A1" t="s" s="35">
         <v>46</v>
       </c>
-      <c r="B1" t="s" s="32">
+      <c r="B1" t="s" s="35">
         <v>60</v>
       </c>
-      <c r="C1" t="s" s="32">
+      <c r="C1" t="s" s="35">
         <v>61</v>
       </c>
-      <c r="D1" t="s" s="32">
+      <c r="D1" t="s" s="35">
         <v>62</v>
       </c>
-      <c r="E1" t="s" s="32">
+      <c r="E1" t="s" s="35">
         <v>63</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>347</v>
+        <v>344</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="D2" t="s" s="0">
         <v>64</v>
@@ -2489,13 +2633,13 @@
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="C3" t="s" s="0">
-        <v>352</v>
+        <v>349</v>
       </c>
       <c r="D3" t="s" s="0">
         <v>64</v>
@@ -2506,13 +2650,13 @@
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="C4" t="s" s="0">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="D4" t="s" s="0">
         <v>64</v>
@@ -2523,13 +2667,13 @@
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>356</v>
+        <v>368</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>357</v>
+        <v>369</v>
       </c>
       <c r="C5" t="s" s="0">
-        <v>358</v>
+        <v>370</v>
       </c>
       <c r="D5" t="s" s="0">
         <v>64</v>
@@ -2540,13 +2684,13 @@
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>359</v>
+        <v>371</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>360</v>
+        <v>372</v>
       </c>
       <c r="C6" t="s" s="0">
-        <v>361</v>
+        <v>373</v>
       </c>
       <c r="D6" t="s" s="0">
         <v>64</v>
@@ -2557,13 +2701,13 @@
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>362</v>
+        <v>569</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>363</v>
+        <v>570</v>
       </c>
       <c r="C7" t="s" s="0">
-        <v>364</v>
+        <v>571</v>
       </c>
       <c r="D7" t="s" s="0">
         <v>64</v>
@@ -2574,13 +2718,13 @@
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>365</v>
+        <v>374</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>366</v>
+        <v>375</v>
       </c>
       <c r="C8" t="s" s="0">
-        <v>367</v>
+        <v>376</v>
       </c>
       <c r="D8" t="s" s="0">
         <v>64</v>
@@ -2591,13 +2735,13 @@
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
-        <v>368</v>
+        <v>377</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>369</v>
+        <v>378</v>
       </c>
       <c r="C9" t="s" s="0">
-        <v>370</v>
+        <v>379</v>
       </c>
       <c r="D9" t="s" s="0">
         <v>64</v>
@@ -2608,13 +2752,13 @@
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
-        <v>371</v>
+        <v>383</v>
       </c>
       <c r="B10" t="s" s="0">
-        <v>372</v>
+        <v>384</v>
       </c>
       <c r="C10" t="s" s="0">
-        <v>373</v>
+        <v>385</v>
       </c>
       <c r="D10" t="s" s="0">
         <v>64</v>
@@ -2625,698 +2769,18 @@
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
-        <v>374</v>
+        <v>386</v>
       </c>
       <c r="B11" t="s" s="0">
-        <v>375</v>
+        <v>387</v>
       </c>
       <c r="C11" t="s" s="0">
-        <v>376</v>
+        <v>388</v>
       </c>
       <c r="D11" t="s" s="0">
         <v>64</v>
       </c>
       <c r="E11" t="s" s="0">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="s" s="0">
-        <v>377</v>
-      </c>
-      <c r="B12" t="s" s="0">
-        <v>378</v>
-      </c>
-      <c r="C12" t="s" s="0">
-        <v>379</v>
-      </c>
-      <c r="D12" t="s" s="0">
-        <v>64</v>
-      </c>
-      <c r="E12" t="s" s="0">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="s" s="0">
-        <v>380</v>
-      </c>
-      <c r="B13" t="s" s="0">
-        <v>381</v>
-      </c>
-      <c r="C13" t="s" s="0">
-        <v>382</v>
-      </c>
-      <c r="D13" t="s" s="0">
-        <v>64</v>
-      </c>
-      <c r="E13" t="s" s="0">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="s" s="0">
-        <v>383</v>
-      </c>
-      <c r="B14" t="s" s="0">
-        <v>384</v>
-      </c>
-      <c r="C14" t="s" s="0">
-        <v>385</v>
-      </c>
-      <c r="D14" t="s" s="0">
-        <v>64</v>
-      </c>
-      <c r="E14" t="s" s="0">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="s" s="0">
-        <v>386</v>
-      </c>
-      <c r="B15" t="s" s="0">
-        <v>387</v>
-      </c>
-      <c r="C15" t="s" s="0">
-        <v>388</v>
-      </c>
-      <c r="D15" t="s" s="0">
-        <v>64</v>
-      </c>
-      <c r="E15" t="s" s="0">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="s" s="0">
-        <v>389</v>
-      </c>
-      <c r="B16" t="s" s="0">
-        <v>390</v>
-      </c>
-      <c r="C16" t="s" s="0">
-        <v>391</v>
-      </c>
-      <c r="D16" t="s" s="0">
-        <v>64</v>
-      </c>
-      <c r="E16" t="s" s="0">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="s" s="0">
-        <v>392</v>
-      </c>
-      <c r="B17" t="s" s="0">
-        <v>393</v>
-      </c>
-      <c r="C17" t="s" s="0">
-        <v>394</v>
-      </c>
-      <c r="D17" t="s" s="0">
-        <v>64</v>
-      </c>
-      <c r="E17" t="s" s="0">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="s" s="0">
-        <v>395</v>
-      </c>
-      <c r="B18" t="s" s="0">
-        <v>396</v>
-      </c>
-      <c r="C18" t="s" s="0">
-        <v>397</v>
-      </c>
-      <c r="D18" t="s" s="0">
-        <v>64</v>
-      </c>
-      <c r="E18" t="s" s="0">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="s" s="0">
-        <v>398</v>
-      </c>
-      <c r="B19" t="s" s="0">
-        <v>399</v>
-      </c>
-      <c r="C19" t="s" s="0">
-        <v>400</v>
-      </c>
-      <c r="D19" t="s" s="0">
-        <v>64</v>
-      </c>
-      <c r="E19" t="s" s="0">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="s" s="0">
-        <v>401</v>
-      </c>
-      <c r="B20" t="s" s="0">
-        <v>402</v>
-      </c>
-      <c r="C20" t="s" s="0">
-        <v>403</v>
-      </c>
-      <c r="D20" t="s" s="0">
-        <v>64</v>
-      </c>
-      <c r="E20" t="s" s="0">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="s" s="0">
-        <v>404</v>
-      </c>
-      <c r="B21" t="s" s="0">
-        <v>405</v>
-      </c>
-      <c r="C21" t="s" s="0">
-        <v>406</v>
-      </c>
-      <c r="D21" t="s" s="0">
-        <v>64</v>
-      </c>
-      <c r="E21" t="s" s="0">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="s" s="0">
-        <v>407</v>
-      </c>
-      <c r="B22" t="s" s="0">
-        <v>408</v>
-      </c>
-      <c r="C22" t="s" s="0">
-        <v>409</v>
-      </c>
-      <c r="D22" t="s" s="0">
-        <v>64</v>
-      </c>
-      <c r="E22" t="s" s="0">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="s" s="0">
-        <v>410</v>
-      </c>
-      <c r="B23" t="s" s="0">
-        <v>411</v>
-      </c>
-      <c r="C23" t="s" s="0">
-        <v>412</v>
-      </c>
-      <c r="D23" t="s" s="0">
-        <v>64</v>
-      </c>
-      <c r="E23" t="s" s="0">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="s" s="0">
-        <v>413</v>
-      </c>
-      <c r="B24" t="s" s="0">
-        <v>414</v>
-      </c>
-      <c r="C24" t="s" s="0">
-        <v>415</v>
-      </c>
-      <c r="D24" t="s" s="0">
-        <v>64</v>
-      </c>
-      <c r="E24" t="s" s="0">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="s" s="0">
-        <v>416</v>
-      </c>
-      <c r="B25" t="s" s="0">
-        <v>417</v>
-      </c>
-      <c r="C25" t="s" s="0">
-        <v>418</v>
-      </c>
-      <c r="D25" t="s" s="0">
-        <v>64</v>
-      </c>
-      <c r="E25" t="s" s="0">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="s" s="0">
-        <v>419</v>
-      </c>
-      <c r="B26" t="s" s="0">
-        <v>420</v>
-      </c>
-      <c r="C26" t="s" s="0">
-        <v>421</v>
-      </c>
-      <c r="D26" t="s" s="0">
-        <v>64</v>
-      </c>
-      <c r="E26" t="s" s="0">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="s" s="0">
-        <v>422</v>
-      </c>
-      <c r="B27" t="s" s="0">
-        <v>423</v>
-      </c>
-      <c r="C27" t="s" s="0">
-        <v>424</v>
-      </c>
-      <c r="D27" t="s" s="0">
-        <v>64</v>
-      </c>
-      <c r="E27" t="s" s="0">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="s" s="0">
-        <v>425</v>
-      </c>
-      <c r="B28" t="s" s="0">
-        <v>426</v>
-      </c>
-      <c r="C28" t="s" s="0">
-        <v>427</v>
-      </c>
-      <c r="D28" t="s" s="0">
-        <v>64</v>
-      </c>
-      <c r="E28" t="s" s="0">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="s" s="0">
-        <v>431</v>
-      </c>
-      <c r="B29" t="s" s="0">
-        <v>432</v>
-      </c>
-      <c r="C29" t="s" s="0">
-        <v>433</v>
-      </c>
-      <c r="D29" t="s" s="0">
-        <v>64</v>
-      </c>
-      <c r="E29" t="s" s="0">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="s" s="0">
-        <v>434</v>
-      </c>
-      <c r="B30" t="s" s="0">
-        <v>435</v>
-      </c>
-      <c r="C30" t="s" s="0">
-        <v>436</v>
-      </c>
-      <c r="D30" t="s" s="0">
-        <v>64</v>
-      </c>
-      <c r="E30" t="s" s="0">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="s" s="0">
-        <v>437</v>
-      </c>
-      <c r="B31" t="s" s="0">
-        <v>438</v>
-      </c>
-      <c r="C31" t="s" s="0">
-        <v>439</v>
-      </c>
-      <c r="D31" t="s" s="0">
-        <v>64</v>
-      </c>
-      <c r="E31" t="s" s="0">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="s" s="0">
-        <v>440</v>
-      </c>
-      <c r="B32" t="s" s="0">
-        <v>441</v>
-      </c>
-      <c r="C32" t="s" s="0">
-        <v>442</v>
-      </c>
-      <c r="D32" t="s" s="0">
-        <v>64</v>
-      </c>
-      <c r="E32" t="s" s="0">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="s" s="0">
-        <v>443</v>
-      </c>
-      <c r="B33" t="s" s="0">
-        <v>444</v>
-      </c>
-      <c r="C33" t="s" s="0">
-        <v>445</v>
-      </c>
-      <c r="D33" t="s" s="0">
-        <v>64</v>
-      </c>
-      <c r="E33" t="s" s="0">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="s" s="0">
-        <v>446</v>
-      </c>
-      <c r="B34" t="s" s="0">
-        <v>447</v>
-      </c>
-      <c r="C34" t="s" s="0">
-        <v>448</v>
-      </c>
-      <c r="D34" t="s" s="0">
-        <v>64</v>
-      </c>
-      <c r="E34" t="s" s="0">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="s" s="0">
-        <v>449</v>
-      </c>
-      <c r="B35" t="s" s="0">
-        <v>450</v>
-      </c>
-      <c r="C35" t="s" s="0">
-        <v>451</v>
-      </c>
-      <c r="D35" t="s" s="0">
-        <v>64</v>
-      </c>
-      <c r="E35" t="s" s="0">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="s" s="0">
-        <v>452</v>
-      </c>
-      <c r="B36" t="s" s="0">
-        <v>453</v>
-      </c>
-      <c r="C36" t="s" s="0">
-        <v>454</v>
-      </c>
-      <c r="D36" t="s" s="0">
-        <v>64</v>
-      </c>
-      <c r="E36" t="s" s="0">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="s" s="0">
-        <v>455</v>
-      </c>
-      <c r="B37" t="s" s="0">
-        <v>456</v>
-      </c>
-      <c r="C37" t="s" s="0">
-        <v>457</v>
-      </c>
-      <c r="D37" t="s" s="0">
-        <v>64</v>
-      </c>
-      <c r="E37" t="s" s="0">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="s" s="0">
-        <v>458</v>
-      </c>
-      <c r="B38" t="s" s="0">
-        <v>459</v>
-      </c>
-      <c r="C38" t="s" s="0">
-        <v>460</v>
-      </c>
-      <c r="D38" t="s" s="0">
-        <v>64</v>
-      </c>
-      <c r="E38" t="s" s="0">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="s" s="0">
-        <v>461</v>
-      </c>
-      <c r="B39" t="s" s="0">
-        <v>462</v>
-      </c>
-      <c r="C39" t="s" s="0">
-        <v>463</v>
-      </c>
-      <c r="D39" t="s" s="0">
-        <v>64</v>
-      </c>
-      <c r="E39" t="s" s="0">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="s" s="0">
-        <v>464</v>
-      </c>
-      <c r="B40" t="s" s="0">
-        <v>465</v>
-      </c>
-      <c r="C40" t="s" s="0">
-        <v>466</v>
-      </c>
-      <c r="D40" t="s" s="0">
-        <v>64</v>
-      </c>
-      <c r="E40" t="s" s="0">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="s" s="0">
-        <v>470</v>
-      </c>
-      <c r="B41" t="s" s="0">
-        <v>471</v>
-      </c>
-      <c r="C41" t="s" s="0">
-        <v>472</v>
-      </c>
-      <c r="D41" t="s" s="0">
-        <v>64</v>
-      </c>
-      <c r="E41" t="s" s="0">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="s" s="0">
-        <v>473</v>
-      </c>
-      <c r="B42" t="s" s="0">
-        <v>474</v>
-      </c>
-      <c r="C42" t="s" s="0">
-        <v>475</v>
-      </c>
-      <c r="D42" t="s" s="0">
-        <v>64</v>
-      </c>
-      <c r="E42" t="s" s="0">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="s" s="0">
-        <v>476</v>
-      </c>
-      <c r="B43" t="s" s="0">
-        <v>477</v>
-      </c>
-      <c r="C43" t="s" s="0">
-        <v>478</v>
-      </c>
-      <c r="D43" t="s" s="0">
-        <v>64</v>
-      </c>
-      <c r="E43" t="s" s="0">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="s" s="0">
-        <v>479</v>
-      </c>
-      <c r="B44" t="s" s="0">
-        <v>480</v>
-      </c>
-      <c r="C44" t="s" s="0">
-        <v>481</v>
-      </c>
-      <c r="D44" t="s" s="0">
-        <v>64</v>
-      </c>
-      <c r="E44" t="s" s="0">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="s" s="0">
-        <v>482</v>
-      </c>
-      <c r="B45" t="s" s="0">
-        <v>483</v>
-      </c>
-      <c r="C45" t="s" s="0">
-        <v>484</v>
-      </c>
-      <c r="D45" t="s" s="0">
-        <v>64</v>
-      </c>
-      <c r="E45" t="s" s="0">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="s" s="0">
-        <v>485</v>
-      </c>
-      <c r="B46" t="s" s="0">
-        <v>486</v>
-      </c>
-      <c r="C46" t="s" s="0">
-        <v>487</v>
-      </c>
-      <c r="D46" t="s" s="0">
-        <v>64</v>
-      </c>
-      <c r="E46" t="s" s="0">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="s" s="0">
-        <v>488</v>
-      </c>
-      <c r="B47" t="s" s="0">
-        <v>489</v>
-      </c>
-      <c r="C47" t="s" s="0">
-        <v>490</v>
-      </c>
-      <c r="D47" t="s" s="0">
-        <v>64</v>
-      </c>
-      <c r="E47" t="s" s="0">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="s" s="0">
-        <v>491</v>
-      </c>
-      <c r="B48" t="s" s="0">
-        <v>492</v>
-      </c>
-      <c r="C48" t="s" s="0">
-        <v>493</v>
-      </c>
-      <c r="D48" t="s" s="0">
-        <v>64</v>
-      </c>
-      <c r="E48" t="s" s="0">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="s" s="0">
-        <v>494</v>
-      </c>
-      <c r="B49" t="s" s="0">
-        <v>495</v>
-      </c>
-      <c r="C49" t="s" s="0">
-        <v>496</v>
-      </c>
-      <c r="D49" t="s" s="0">
-        <v>64</v>
-      </c>
-      <c r="E49" t="s" s="0">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="s" s="0">
-        <v>497</v>
-      </c>
-      <c r="B50" t="s" s="0">
-        <v>498</v>
-      </c>
-      <c r="C50" t="s" s="0">
-        <v>499</v>
-      </c>
-      <c r="D50" t="s" s="0">
-        <v>64</v>
-      </c>
-      <c r="E50" t="s" s="0">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="s" s="0">
-        <v>500</v>
-      </c>
-      <c r="B51" t="s" s="0">
-        <v>501</v>
-      </c>
-      <c r="C51" t="s" s="0">
-        <v>502</v>
-      </c>
-      <c r="D51" t="s" s="0">
-        <v>64</v>
-      </c>
-      <c r="E51" t="s" s="0">
         <v>65</v>
       </c>
     </row>

</xml_diff>